<commit_message>
data: refresh source state (2026-10-27)
</commit_message>
<xml_diff>
--- a/data/raw/gadoe_revenues_2025.xlsx
+++ b/data/raw/gadoe_revenues_2025.xlsx
@@ -485,7 +485,7 @@
         </is>
       </c>
       <c s="6" r="D11">
-        <v>3266</v>
+        <v>3266.00</v>
       </c>
       <c s="7" r="E11">
         <v>18751117.94</v>
@@ -533,13 +533,13 @@
         </is>
       </c>
       <c s="6" r="D12">
-        <v>1557</v>
+        <v>1557.00</v>
       </c>
       <c s="7" r="E12">
         <v>3570825.33</v>
       </c>
       <c s="7" r="F12">
-        <v>2293.4</v>
+        <v>2293.40</v>
       </c>
       <c s="7" r="G12">
         <v>16.14</v>
@@ -581,13 +581,13 @@
         </is>
       </c>
       <c s="6" r="D13">
-        <v>2067</v>
+        <v>2067.00</v>
       </c>
       <c s="7" r="E13">
         <v>6679507.34</v>
       </c>
       <c s="7" r="F13">
-        <v>3231.5</v>
+        <v>3231.50</v>
       </c>
       <c s="7" r="G13">
         <v>21.46</v>
@@ -602,7 +602,7 @@
         <v>70.29</v>
       </c>
       <c s="7" r="K13">
-        <v>2565223</v>
+        <v>2565223.00</v>
       </c>
       <c s="7" r="L13">
         <v>1241.04</v>
@@ -611,7 +611,7 @@
         <v>8.24</v>
       </c>
       <c s="7" r="N13">
-        <v>31118725.5</v>
+        <v>31118725.50</v>
       </c>
       <c s="7" r="O13">
         <v>15055.02</v>
@@ -629,13 +629,13 @@
         </is>
       </c>
       <c s="6" r="D14">
-        <v>277</v>
+        <v>277.00</v>
       </c>
       <c s="7" r="E14">
         <v>2533164.46</v>
       </c>
       <c s="7" r="F14">
-        <v>9145</v>
+        <v>9145.00</v>
       </c>
       <c s="7" r="G14">
         <v>37.43</v>
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c s="6" r="D15">
-        <v>4244</v>
+        <v>4244.00</v>
       </c>
       <c s="7" r="E15">
         <v>24086072.35</v>
@@ -686,10 +686,10 @@
         <v>5675.32</v>
       </c>
       <c s="7" r="G15">
-        <v>38.9</v>
+        <v>38.90</v>
       </c>
       <c s="7" r="H15">
-        <v>30188577.2</v>
+        <v>30188577.20</v>
       </c>
       <c s="7" r="I15">
         <v>7113.24</v>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c s="6" r="D16">
-        <v>2835</v>
+        <v>2835.00</v>
       </c>
       <c s="7" r="E16">
         <v>19552201.62</v>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c s="6" r="D17">
-        <v>15468</v>
+        <v>15468.00</v>
       </c>
       <c s="7" r="E17">
         <v>84347109.58</v>
@@ -791,13 +791,13 @@
         <v>8490.57</v>
       </c>
       <c s="7" r="J17">
-        <v>57.4</v>
+        <v>57.40</v>
       </c>
       <c s="7" r="K17">
         <v>13140067.13</v>
       </c>
       <c s="7" r="L17">
-        <v>849.5</v>
+        <v>849.50</v>
       </c>
       <c s="7" r="M17">
         <v>5.74</v>
@@ -821,7 +821,7 @@
         </is>
       </c>
       <c s="6" r="D18">
-        <v>13788</v>
+        <v>13788.00</v>
       </c>
       <c s="7" r="E18">
         <v>112324661.46</v>
@@ -848,7 +848,7 @@
         <v>1101.92</v>
       </c>
       <c s="7" r="M18">
-        <v>6.7</v>
+        <v>6.70</v>
       </c>
       <c s="7" r="N18">
         <v>226855124.41</v>
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c s="6" r="D19">
-        <v>2640</v>
+        <v>2640.00</v>
       </c>
       <c s="7" r="E19">
         <v>9297494.97</v>
@@ -878,7 +878,7 @@
         <v>3521.78</v>
       </c>
       <c s="7" r="G19">
-        <v>21.1</v>
+        <v>21.10</v>
       </c>
       <c s="7" r="H19">
         <v>30734192.62</v>
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c s="6" r="D20">
-        <v>2945</v>
+        <v>2945.00</v>
       </c>
       <c s="7" r="E20">
         <v>8562272.52</v>
@@ -965,10 +965,10 @@
         </is>
       </c>
       <c s="6" r="D21">
-        <v>20784</v>
+        <v>20784.00</v>
       </c>
       <c s="7" r="E21">
-        <v>106756446.6</v>
+        <v>106756446.60</v>
       </c>
       <c s="7" r="F21">
         <v>5136.47</v>
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c s="6" r="D22">
-        <v>2453</v>
+        <v>2453.00</v>
       </c>
       <c s="7" r="E22">
         <v>6197619.64</v>
@@ -1046,7 +1046,7 @@
         <v>35679371.37</v>
       </c>
       <c s="7" r="O22">
-        <v>14545.2</v>
+        <v>14545.20</v>
       </c>
     </row>
     <row r="23" ht="14.4" customHeight="0">
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c s="6" r="D23">
-        <v>3209</v>
+        <v>3209.00</v>
       </c>
       <c s="7" r="E23">
         <v>7531548.22</v>
@@ -1076,13 +1076,13 @@
         <v>34653017.86</v>
       </c>
       <c s="7" r="I23">
-        <v>10798.7</v>
+        <v>10798.70</v>
       </c>
       <c s="7" r="J23">
         <v>76.42</v>
       </c>
       <c s="7" r="K23">
-        <v>3162581</v>
+        <v>3162581.00</v>
       </c>
       <c s="7" r="L23">
         <v>985.53</v>
@@ -1109,10 +1109,10 @@
         </is>
       </c>
       <c s="6" r="D24">
-        <v>2159</v>
+        <v>2159.00</v>
       </c>
       <c s="7" r="E24">
-        <v>10390336.1</v>
+        <v>10390336.10</v>
       </c>
       <c s="7" r="F24">
         <v>4812.57</v>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c s="6" r="D25">
-        <v>10439</v>
+        <v>10439.00</v>
       </c>
       <c s="7" r="E25">
         <v>52790764.72</v>
@@ -1205,19 +1205,19 @@
         </is>
       </c>
       <c s="6" r="D26">
-        <v>10610</v>
+        <v>10610.00</v>
       </c>
       <c s="7" r="E26">
         <v>58245764.09</v>
       </c>
       <c s="7" r="F26">
-        <v>5489.7</v>
+        <v>5489.70</v>
       </c>
       <c s="7" r="G26">
         <v>36.19</v>
       </c>
       <c s="7" r="H26">
-        <v>94577691.8</v>
+        <v>94577691.80</v>
       </c>
       <c s="7" r="I26">
         <v>8914.01</v>
@@ -1253,7 +1253,7 @@
         </is>
       </c>
       <c s="6" r="D27">
-        <v>3626</v>
+        <v>3626.00</v>
       </c>
       <c s="7" r="E27">
         <v>128902048.16</v>
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c s="6" r="D28">
-        <v>3361</v>
+        <v>3361.00</v>
       </c>
       <c s="7" r="E28">
         <v>23122172.52</v>
@@ -1331,7 +1331,7 @@
         <v>8.22</v>
       </c>
       <c s="7" r="N28">
-        <v>52894719.1</v>
+        <v>52894719.10</v>
       </c>
       <c s="7" r="O28">
         <v>15737.79</v>
@@ -1349,7 +1349,7 @@
         </is>
       </c>
       <c s="6" r="D29">
-        <v>433</v>
+        <v>433.00</v>
       </c>
       <c s="7" r="E29">
         <v>3375439.89</v>
@@ -1397,7 +1397,7 @@
         </is>
       </c>
       <c s="6" r="D30">
-        <v>9563</v>
+        <v>9563.00</v>
       </c>
       <c s="7" r="E30">
         <v>40593645.83</v>
@@ -1430,7 +1430,7 @@
         <v>129211332.53</v>
       </c>
       <c s="7" r="O30">
-        <v>13511.6</v>
+        <v>13511.60</v>
       </c>
     </row>
     <row r="31" ht="14.4" customHeight="0">
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c s="6" r="D31">
-        <v>2051</v>
+        <v>2051.00</v>
       </c>
       <c s="7" r="E31">
         <v>7083434.17</v>
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c s="6" r="D32">
-        <v>15981</v>
+        <v>15981.00</v>
       </c>
       <c s="7" r="E32">
         <v>74406295.05</v>
@@ -1523,7 +1523,7 @@
         <v>5.25</v>
       </c>
       <c s="7" r="N32">
-        <v>223478012.6</v>
+        <v>223478012.60</v>
       </c>
       <c s="7" r="O32">
         <v>13983.98</v>
@@ -1541,10 +1541,10 @@
         </is>
       </c>
       <c s="6" r="D33">
-        <v>9890</v>
+        <v>9890.00</v>
       </c>
       <c s="7" r="E33">
-        <v>53340213.4</v>
+        <v>53340213.40</v>
       </c>
       <c s="7" r="F33">
         <v>5393.35</v>
@@ -1589,7 +1589,7 @@
         </is>
       </c>
       <c s="6" r="D34">
-        <v>1525</v>
+        <v>1525.00</v>
       </c>
       <c s="7" r="E34">
         <v>6726637.51</v>
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c s="6" r="D35">
-        <v>34915</v>
+        <v>34915.00</v>
       </c>
       <c s="7" r="E35">
         <v>436072910.02</v>
@@ -1685,7 +1685,7 @@
         </is>
       </c>
       <c s="6" r="D36">
-        <v>921</v>
+        <v>921.00</v>
       </c>
       <c s="7" r="E36">
         <v>2295056.92</v>
@@ -1703,13 +1703,13 @@
         <v>12083.57</v>
       </c>
       <c s="7" r="J36">
-        <v>67.1</v>
+        <v>67.10</v>
       </c>
       <c s="7" r="K36">
         <v>3161053.37</v>
       </c>
       <c s="7" r="L36">
-        <v>3432.2</v>
+        <v>3432.20</v>
       </c>
       <c s="7" r="M36">
         <v>19.06</v>
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c s="6" r="D37">
-        <v>2592</v>
+        <v>2592.00</v>
       </c>
       <c s="7" r="E37">
         <v>11682236.83</v>
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c s="6" r="D38">
-        <v>43079</v>
+        <v>43079.00</v>
       </c>
       <c s="7" r="E38">
         <v>312811039.54</v>
@@ -1790,7 +1790,7 @@
         <v>7261.33</v>
       </c>
       <c s="7" r="G38">
-        <v>50</v>
+        <v>50.00</v>
       </c>
       <c s="7" r="H38">
         <v>296052217.05</v>
@@ -1802,7 +1802,7 @@
         <v>47.32</v>
       </c>
       <c s="7" r="K38">
-        <v>16727154.1</v>
+        <v>16727154.10</v>
       </c>
       <c s="7" r="L38">
         <v>388.29</v>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c s="6" r="D39">
-        <v>12135</v>
+        <v>12135.00</v>
       </c>
       <c s="7" r="E39">
         <v>151134977.81</v>
@@ -1877,7 +1877,7 @@
         </is>
       </c>
       <c s="6" r="D40">
-        <v>173</v>
+        <v>173.00</v>
       </c>
       <c s="7" r="E40">
         <v>1851716.74</v>
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c s="6" r="D41">
-        <v>51724</v>
+        <v>51724.00</v>
       </c>
       <c s="7" r="E41">
         <v>267928111.55</v>
@@ -1958,7 +1958,7 @@
         <v>772415384.67</v>
       </c>
       <c s="7" r="O41">
-        <v>14933.4</v>
+        <v>14933.40</v>
       </c>
     </row>
     <row r="42" ht="14.4" customHeight="0">
@@ -1973,10 +1973,10 @@
         </is>
       </c>
       <c s="6" r="D42">
-        <v>1173</v>
+        <v>1173.00</v>
       </c>
       <c s="7" r="E42">
-        <v>6184097</v>
+        <v>6184097.00</v>
       </c>
       <c s="7" r="F42">
         <v>5272.03</v>
@@ -2003,7 +2003,7 @@
         <v>7.21</v>
       </c>
       <c s="7" r="N42">
-        <v>19916975.4</v>
+        <v>19916975.40</v>
       </c>
       <c s="7" r="O42">
         <v>16979.51</v>
@@ -2021,10 +2021,10 @@
         </is>
       </c>
       <c s="6" r="D43">
-        <v>109011</v>
+        <v>109011.00</v>
       </c>
       <c s="7" r="E43">
-        <v>895759146.9</v>
+        <v>895759146.90</v>
       </c>
       <c s="7" r="F43">
         <v>8217.14</v>
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c s="6" r="D44">
-        <v>7450</v>
+        <v>7450.00</v>
       </c>
       <c s="7" r="E44">
         <v>20669404.09</v>
@@ -2099,7 +2099,7 @@
         <v>10.12</v>
       </c>
       <c s="7" r="N44">
-        <v>104214508.1</v>
+        <v>104214508.10</v>
       </c>
       <c s="7" r="O44">
         <v>13988.53</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c s="6" r="D45">
-        <v>8778</v>
+        <v>8778.00</v>
       </c>
       <c s="7" r="E45">
         <v>26861094.13</v>
@@ -2150,7 +2150,7 @@
         <v>137613593.41</v>
       </c>
       <c s="7" r="O45">
-        <v>15677.1</v>
+        <v>15677.10</v>
       </c>
     </row>
     <row r="46" ht="14.4" customHeight="0">
@@ -2165,7 +2165,7 @@
         </is>
       </c>
       <c s="6" r="D46">
-        <v>28626</v>
+        <v>28626.00</v>
       </c>
       <c s="7" r="E46">
         <v>157259406.04</v>
@@ -2213,7 +2213,7 @@
         </is>
       </c>
       <c s="6" r="D47">
-        <v>2867</v>
+        <v>2867.00</v>
       </c>
       <c s="7" r="E47">
         <v>9296068.68</v>
@@ -2261,7 +2261,7 @@
         </is>
       </c>
       <c s="6" r="D48">
-        <v>22759</v>
+        <v>22759.00</v>
       </c>
       <c s="7" r="E48">
         <v>162731951.62</v>
@@ -2309,10 +2309,10 @@
         </is>
       </c>
       <c s="6" r="D49">
-        <v>1470</v>
+        <v>1470.00</v>
       </c>
       <c s="7" r="E49">
-        <v>7795002</v>
+        <v>7795002.00</v>
       </c>
       <c s="7" r="F49">
         <v>5302.72</v>
@@ -2357,7 +2357,7 @@
         </is>
       </c>
       <c s="6" r="D50">
-        <v>3117</v>
+        <v>3117.00</v>
       </c>
       <c s="7" r="E50">
         <v>14100000.38</v>
@@ -2366,7 +2366,7 @@
         <v>4523.58</v>
       </c>
       <c s="7" r="G50">
-        <v>27</v>
+        <v>27.00</v>
       </c>
       <c s="7" r="H50">
         <v>31272368.84</v>
@@ -2405,7 +2405,7 @@
         </is>
       </c>
       <c s="6" r="D51">
-        <v>1885</v>
+        <v>1885.00</v>
       </c>
       <c s="7" r="E51">
         <v>9785723.29</v>
@@ -2426,7 +2426,7 @@
         <v>57.31</v>
       </c>
       <c s="7" r="K51">
-        <v>1480407.6</v>
+        <v>1480407.60</v>
       </c>
       <c s="7" r="L51">
         <v>785.36</v>
@@ -2453,10 +2453,10 @@
         </is>
       </c>
       <c s="6" r="D52">
-        <v>4258</v>
+        <v>4258.00</v>
       </c>
       <c s="7" r="E52">
-        <v>35084583.6</v>
+        <v>35084583.60</v>
       </c>
       <c s="7" r="F52">
         <v>8239.69</v>
@@ -2465,7 +2465,7 @@
         <v>54.54</v>
       </c>
       <c s="7" r="H52">
-        <v>27413382.5</v>
+        <v>27413382.50</v>
       </c>
       <c s="7" r="I52">
         <v>6438.09</v>
@@ -2477,7 +2477,7 @@
         <v>1829674.37</v>
       </c>
       <c s="7" r="L52">
-        <v>429.7</v>
+        <v>429.70</v>
       </c>
       <c s="7" r="M52">
         <v>2.84</v>
@@ -2501,7 +2501,7 @@
         </is>
       </c>
       <c s="6" r="D53">
-        <v>4010</v>
+        <v>4010.00</v>
       </c>
       <c s="7" r="E53">
         <v>20421995.93</v>
@@ -2549,7 +2549,7 @@
         </is>
       </c>
       <c s="6" r="D54">
-        <v>93513</v>
+        <v>93513.00</v>
       </c>
       <c s="7" r="E54">
         <v>1010115796.99</v>
@@ -2573,7 +2573,7 @@
         <v>190336118.82</v>
       </c>
       <c s="7" r="L54">
-        <v>2035.4</v>
+        <v>2035.40</v>
       </c>
       <c s="7" r="M54">
         <v>10.35</v>
@@ -2582,7 +2582,7 @@
         <v>1839642821.28</v>
       </c>
       <c s="7" r="O54">
-        <v>19672.6</v>
+        <v>19672.60</v>
       </c>
     </row>
     <row r="55" ht="14.4" customHeight="0">
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c s="6" r="D55">
-        <v>2580</v>
+        <v>2580.00</v>
       </c>
       <c s="7" r="E55">
         <v>8340180.06</v>
@@ -2645,7 +2645,7 @@
         </is>
       </c>
       <c s="6" r="D56">
-        <v>1045</v>
+        <v>1045.00</v>
       </c>
       <c s="7" r="E56">
         <v>9120169.26</v>
@@ -2657,7 +2657,7 @@
         <v>41.15</v>
       </c>
       <c s="7" r="H56">
-        <v>9279578.9</v>
+        <v>9279578.90</v>
       </c>
       <c s="7" r="I56">
         <v>8879.98</v>
@@ -2675,7 +2675,7 @@
         <v>16.98</v>
       </c>
       <c s="7" r="N56">
-        <v>22161755.8</v>
+        <v>22161755.80</v>
       </c>
       <c s="7" r="O56">
         <v>21207.42</v>
@@ -2693,7 +2693,7 @@
         </is>
       </c>
       <c s="6" r="D57">
-        <v>12526</v>
+        <v>12526.00</v>
       </c>
       <c s="7" r="E57">
         <v>52955996.05</v>
@@ -2717,7 +2717,7 @@
         <v>28355073.18</v>
       </c>
       <c s="7" r="L57">
-        <v>2263.7</v>
+        <v>2263.70</v>
       </c>
       <c s="7" r="M57">
         <v>13.57</v>
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c s="6" r="D58">
-        <v>25849</v>
+        <v>25849.00</v>
       </c>
       <c s="7" r="E58">
         <v>146530791.63</v>
@@ -2756,7 +2756,7 @@
         <v>191815143.62</v>
       </c>
       <c s="7" r="I58">
-        <v>7420.6</v>
+        <v>7420.60</v>
       </c>
       <c s="7" r="J58">
         <v>53.05</v>
@@ -2789,13 +2789,13 @@
         </is>
       </c>
       <c s="6" r="D59">
-        <v>1426</v>
+        <v>1426.00</v>
       </c>
       <c s="7" r="E59">
         <v>9395490.87</v>
       </c>
       <c s="7" r="F59">
-        <v>6588.7</v>
+        <v>6588.70</v>
       </c>
       <c s="7" r="G59">
         <v>37.41</v>
@@ -2816,7 +2816,7 @@
         <v>1761.93</v>
       </c>
       <c s="7" r="M59">
-        <v>10</v>
+        <v>10.00</v>
       </c>
       <c s="7" r="N59">
         <v>25115935.85</v>
@@ -2837,7 +2837,7 @@
         </is>
       </c>
       <c s="6" r="D60">
-        <v>917</v>
+        <v>917.00</v>
       </c>
       <c s="7" r="E60">
         <v>2498132.18</v>
@@ -2855,7 +2855,7 @@
         <v>10419.27</v>
       </c>
       <c s="7" r="J60">
-        <v>73.2</v>
+        <v>73.20</v>
       </c>
       <c s="7" r="K60">
         <v>999683.42</v>
@@ -2885,10 +2885,10 @@
         </is>
       </c>
       <c s="6" r="D61">
-        <v>14067</v>
+        <v>14067.00</v>
       </c>
       <c s="7" r="E61">
-        <v>71844764.4</v>
+        <v>71844764.40</v>
       </c>
       <c s="7" r="F61">
         <v>5107.33</v>
@@ -2900,7 +2900,7 @@
         <v>120399396.17</v>
       </c>
       <c s="7" r="I61">
-        <v>8559</v>
+        <v>8559.00</v>
       </c>
       <c s="7" r="J61">
         <v>60.65</v>
@@ -2933,7 +2933,7 @@
         </is>
       </c>
       <c s="6" r="D62">
-        <v>2887</v>
+        <v>2887.00</v>
       </c>
       <c s="7" r="E62">
         <v>14332734.55</v>
@@ -2981,10 +2981,10 @@
         </is>
       </c>
       <c s="6" r="D63">
-        <v>3768</v>
+        <v>3768.00</v>
       </c>
       <c s="7" r="E63">
-        <v>10832504.4</v>
+        <v>10832504.40</v>
       </c>
       <c s="7" r="F63">
         <v>2874.87</v>
@@ -2993,7 +2993,7 @@
         <v>19.06</v>
       </c>
       <c s="7" r="H63">
-        <v>39432696.7</v>
+        <v>39432696.70</v>
       </c>
       <c s="7" r="I63">
         <v>10465.15</v>
@@ -3029,7 +3029,7 @@
         </is>
       </c>
       <c s="6" r="D64">
-        <v>1733</v>
+        <v>1733.00</v>
       </c>
       <c s="7" r="E64">
         <v>5858264.03</v>
@@ -3041,10 +3041,10 @@
         <v>21.44</v>
       </c>
       <c s="7" r="H64">
-        <v>19071497.6</v>
+        <v>19071497.60</v>
       </c>
       <c s="7" r="I64">
-        <v>11004.9</v>
+        <v>11004.90</v>
       </c>
       <c s="7" r="J64">
         <v>69.81</v>
@@ -3077,7 +3077,7 @@
         </is>
       </c>
       <c s="6" r="D65">
-        <v>2682</v>
+        <v>2682.00</v>
       </c>
       <c s="7" r="E65">
         <v>29035010.17</v>
@@ -3110,7 +3110,7 @@
         <v>44981178.51</v>
       </c>
       <c s="7" r="O65">
-        <v>16771.5</v>
+        <v>16771.50</v>
       </c>
     </row>
     <row r="66" ht="14.4" customHeight="0">
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c s="6" r="D66">
-        <v>19849</v>
+        <v>19849.00</v>
       </c>
       <c s="7" r="E66">
         <v>156280503.55</v>
@@ -3155,7 +3155,7 @@
         <v>2.65</v>
       </c>
       <c s="7" r="N66">
-        <v>302790998.1</v>
+        <v>302790998.10</v>
       </c>
       <c s="7" r="O66">
         <v>15254.73</v>
@@ -3173,7 +3173,7 @@
         </is>
       </c>
       <c s="6" r="D67">
-        <v>8682</v>
+        <v>8682.00</v>
       </c>
       <c s="7" r="E67">
         <v>60613111.77</v>
@@ -3197,7 +3197,7 @@
         <v>6964706.29</v>
       </c>
       <c s="7" r="L67">
-        <v>802.2</v>
+        <v>802.20</v>
       </c>
       <c s="7" r="M67">
         <v>4.75</v>
@@ -3221,7 +3221,7 @@
         </is>
       </c>
       <c s="6" r="D68">
-        <v>55313</v>
+        <v>55313.00</v>
       </c>
       <c s="7" r="E68">
         <v>385716325.41</v>
@@ -3230,7 +3230,7 @@
         <v>6973.34</v>
       </c>
       <c s="7" r="G68">
-        <v>51.9</v>
+        <v>51.90</v>
       </c>
       <c s="7" r="H68">
         <v>343157458.27</v>
@@ -3245,7 +3245,7 @@
         <v>14287270.23</v>
       </c>
       <c s="7" r="L68">
-        <v>258.3</v>
+        <v>258.30</v>
       </c>
       <c s="7" r="M68">
         <v>1.92</v>
@@ -3269,7 +3269,7 @@
         </is>
       </c>
       <c s="6" r="D69">
-        <v>3604</v>
+        <v>3604.00</v>
       </c>
       <c s="7" r="E69">
         <v>18504779.37</v>
@@ -3317,7 +3317,7 @@
         </is>
       </c>
       <c s="6" r="D70">
-        <v>86863</v>
+        <v>86863.00</v>
       </c>
       <c s="7" r="E70">
         <v>909199909.94</v>
@@ -3365,13 +3365,13 @@
         </is>
       </c>
       <c s="6" r="D71">
-        <v>4174</v>
+        <v>4174.00</v>
       </c>
       <c s="7" r="E71">
         <v>28015071.69</v>
       </c>
       <c s="7" r="F71">
-        <v>6711.8</v>
+        <v>6711.80</v>
       </c>
       <c s="7" r="G71">
         <v>47.15</v>
@@ -3413,7 +3413,7 @@
         </is>
       </c>
       <c s="6" r="D72">
-        <v>548</v>
+        <v>548.00</v>
       </c>
       <c s="7" r="E72">
         <v>1850298.27</v>
@@ -3425,10 +3425,10 @@
         <v>19.45</v>
       </c>
       <c s="7" r="H72">
-        <v>6091019</v>
+        <v>6091019.00</v>
       </c>
       <c s="7" r="I72">
-        <v>11115</v>
+        <v>11115.00</v>
       </c>
       <c s="7" r="J72">
         <v>64.03</v>
@@ -3461,7 +3461,7 @@
         </is>
       </c>
       <c s="6" r="D73">
-        <v>12701</v>
+        <v>12701.00</v>
       </c>
       <c s="7" r="E73">
         <v>110192202.86</v>
@@ -3482,7 +3482,7 @@
         <v>38.25</v>
       </c>
       <c s="7" r="K73">
-        <v>13262771</v>
+        <v>13262771.00</v>
       </c>
       <c s="7" r="L73">
         <v>1044.23</v>
@@ -3509,7 +3509,7 @@
         </is>
       </c>
       <c s="6" r="D74">
-        <v>6104</v>
+        <v>6104.00</v>
       </c>
       <c s="7" r="E74">
         <v>26942227.04</v>
@@ -3557,7 +3557,7 @@
         </is>
       </c>
       <c s="6" r="D75">
-        <v>4381</v>
+        <v>4381.00</v>
       </c>
       <c s="7" r="E75">
         <v>13367483.23</v>
@@ -3605,7 +3605,7 @@
         </is>
       </c>
       <c s="6" r="D76">
-        <v>2473</v>
+        <v>2473.00</v>
       </c>
       <c s="7" r="E76">
         <v>37119572.85</v>
@@ -3653,7 +3653,7 @@
         </is>
       </c>
       <c s="6" r="D77">
-        <v>192811</v>
+        <v>192811.00</v>
       </c>
       <c s="7" r="E77">
         <v>1226408596.84</v>
@@ -3701,7 +3701,7 @@
         </is>
       </c>
       <c s="6" r="D78">
-        <v>7361</v>
+        <v>7361.00</v>
       </c>
       <c s="7" r="E78">
         <v>35883993.72</v>
@@ -3710,13 +3710,13 @@
         <v>4874.88</v>
       </c>
       <c s="7" r="G78">
-        <v>33.3</v>
+        <v>33.30</v>
       </c>
       <c s="7" r="H78">
         <v>66966664.27</v>
       </c>
       <c s="7" r="I78">
-        <v>9097.5</v>
+        <v>9097.50</v>
       </c>
       <c s="7" r="J78">
         <v>62.14</v>
@@ -3734,7 +3734,7 @@
         <v>107767944.43</v>
       </c>
       <c s="7" r="O78">
-        <v>14640.4</v>
+        <v>14640.40</v>
       </c>
     </row>
     <row r="79" ht="14.4" customHeight="0">
@@ -3749,7 +3749,7 @@
         </is>
       </c>
       <c s="6" r="D79">
-        <v>28665</v>
+        <v>28665.00</v>
       </c>
       <c s="7" r="E79">
         <v>169264747.66</v>
@@ -3758,13 +3758,13 @@
         <v>5904.93</v>
       </c>
       <c s="7" r="G79">
-        <v>44</v>
+        <v>44.00</v>
       </c>
       <c s="7" r="H79">
         <v>194833064.81</v>
       </c>
       <c s="7" r="I79">
-        <v>6796.9</v>
+        <v>6796.90</v>
       </c>
       <c s="7" r="J79">
         <v>50.65</v>
@@ -3797,7 +3797,7 @@
         </is>
       </c>
       <c s="6" r="D80">
-        <v>628</v>
+        <v>628.00</v>
       </c>
       <c s="7" r="E80">
         <v>6057918.09</v>
@@ -3809,7 +3809,7 @@
         <v>44.72</v>
       </c>
       <c s="7" r="H80">
-        <v>5059614.5</v>
+        <v>5059614.50</v>
       </c>
       <c s="7" r="I80">
         <v>8056.71</v>
@@ -3845,7 +3845,7 @@
         </is>
       </c>
       <c s="6" r="D81">
-        <v>3375</v>
+        <v>3375.00</v>
       </c>
       <c s="7" r="E81">
         <v>15353321.28</v>
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c s="6" r="D82">
-        <v>5418</v>
+        <v>5418.00</v>
       </c>
       <c s="7" r="E82">
         <v>34240442.62</v>
@@ -3941,7 +3941,7 @@
         </is>
       </c>
       <c s="6" r="D83">
-        <v>3653</v>
+        <v>3653.00</v>
       </c>
       <c s="7" r="E83">
         <v>20565493.13</v>
@@ -3989,7 +3989,7 @@
         </is>
       </c>
       <c s="6" r="D84">
-        <v>2118</v>
+        <v>2118.00</v>
       </c>
       <c s="7" r="E84">
         <v>10527396.73</v>
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c s="6" r="D85">
-        <v>43144</v>
+        <v>43144.00</v>
       </c>
       <c s="7" r="E85">
         <v>294468949.43</v>
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c s="6" r="D86">
-        <v>30159</v>
+        <v>30159.00</v>
       </c>
       <c s="7" r="E86">
         <v>134970789.02</v>
@@ -4133,10 +4133,10 @@
         </is>
       </c>
       <c s="6" r="D87">
-        <v>1528</v>
+        <v>1528.00</v>
       </c>
       <c s="7" r="E87">
-        <v>5054509.1</v>
+        <v>5054509.10</v>
       </c>
       <c s="7" r="F87">
         <v>3307.92</v>
@@ -4148,7 +4148,7 @@
         <v>17982727.36</v>
       </c>
       <c s="7" r="I87">
-        <v>11768.8</v>
+        <v>11768.80</v>
       </c>
       <c s="7" r="J87">
         <v>73.36</v>
@@ -4181,7 +4181,7 @@
         </is>
       </c>
       <c s="6" r="D88">
-        <v>11132</v>
+        <v>11132.00</v>
       </c>
       <c s="7" r="E88">
         <v>79577687.21</v>
@@ -4205,13 +4205,13 @@
         <v>5156383.51</v>
       </c>
       <c s="7" r="L88">
-        <v>463.2</v>
+        <v>463.20</v>
       </c>
       <c s="7" r="M88">
         <v>3.02</v>
       </c>
       <c s="7" r="N88">
-        <v>170533526.8</v>
+        <v>170533526.80</v>
       </c>
       <c s="7" r="O88">
         <v>15319.21</v>
@@ -4229,7 +4229,7 @@
         </is>
       </c>
       <c s="6" r="D89">
-        <v>2622</v>
+        <v>2622.00</v>
       </c>
       <c s="7" r="E89">
         <v>12711211.43</v>
@@ -4277,10 +4277,10 @@
         </is>
       </c>
       <c s="6" r="D90">
-        <v>2957</v>
+        <v>2957.00</v>
       </c>
       <c s="7" r="E90">
-        <v>10236859.7</v>
+        <v>10236859.70</v>
       </c>
       <c s="7" r="F90">
         <v>3461.91</v>
@@ -4292,7 +4292,7 @@
         <v>28356458.81</v>
       </c>
       <c s="7" r="I90">
-        <v>9589.6</v>
+        <v>9589.60</v>
       </c>
       <c s="7" r="J90">
         <v>69.18</v>
@@ -4307,7 +4307,7 @@
         <v>5.85</v>
       </c>
       <c s="7" r="N90">
-        <v>40991299.2</v>
+        <v>40991299.20</v>
       </c>
       <c s="7" r="O90">
         <v>13862.46</v>
@@ -4325,7 +4325,7 @@
         </is>
       </c>
       <c s="6" r="D91">
-        <v>1941</v>
+        <v>1941.00</v>
       </c>
       <c s="7" r="E91">
         <v>11572841.02</v>
@@ -4373,7 +4373,7 @@
         </is>
       </c>
       <c s="6" r="D92">
-        <v>1695</v>
+        <v>1695.00</v>
       </c>
       <c s="7" r="E92">
         <v>5372595.65</v>
@@ -4382,7 +4382,7 @@
         <v>3169.67</v>
       </c>
       <c s="7" r="G92">
-        <v>25.4</v>
+        <v>25.40</v>
       </c>
       <c s="7" r="H92">
         <v>14114514.76</v>
@@ -4421,7 +4421,7 @@
         </is>
       </c>
       <c s="6" r="D93">
-        <v>991</v>
+        <v>991.00</v>
       </c>
       <c s="7" r="E93">
         <v>4835422.63</v>
@@ -4469,7 +4469,7 @@
         </is>
       </c>
       <c s="6" r="D94">
-        <v>4788</v>
+        <v>4788.00</v>
       </c>
       <c s="7" r="E94">
         <v>17762149.84</v>
@@ -4517,7 +4517,7 @@
         </is>
       </c>
       <c s="6" r="D95">
-        <v>2772</v>
+        <v>2772.00</v>
       </c>
       <c s="7" r="E95">
         <v>12907440.44</v>
@@ -4529,7 +4529,7 @@
         <v>33.56</v>
       </c>
       <c s="7" r="H95">
-        <v>21707468.9</v>
+        <v>21707468.90</v>
       </c>
       <c s="7" r="I95">
         <v>7830.98</v>
@@ -4547,7 +4547,7 @@
         <v>9.99</v>
       </c>
       <c s="7" r="N95">
-        <v>38456825.2</v>
+        <v>38456825.20</v>
       </c>
       <c s="7" r="O95">
         <v>13873.31</v>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c s="6" r="D96">
-        <v>1560</v>
+        <v>1560.00</v>
       </c>
       <c s="7" r="E96">
         <v>5424757.13</v>
@@ -4613,10 +4613,10 @@
         </is>
       </c>
       <c s="6" r="D97">
-        <v>6070</v>
+        <v>6070.00</v>
       </c>
       <c s="7" r="E97">
-        <v>20976253.5</v>
+        <v>20976253.50</v>
       </c>
       <c s="7" r="F97">
         <v>3455.73</v>
@@ -4634,7 +4634,7 @@
         <v>70.36</v>
       </c>
       <c s="7" r="K97">
-        <v>4953192</v>
+        <v>4953192.00</v>
       </c>
       <c s="7" r="L97">
         <v>816.01</v>
@@ -4661,7 +4661,7 @@
         </is>
       </c>
       <c s="6" r="D98">
-        <v>5733</v>
+        <v>5733.00</v>
       </c>
       <c s="7" r="E98">
         <v>24092871.65</v>
@@ -4709,7 +4709,7 @@
         </is>
       </c>
       <c s="6" r="D99">
-        <v>10592</v>
+        <v>10592.00</v>
       </c>
       <c s="7" r="E99">
         <v>34127490.33</v>
@@ -4739,7 +4739,7 @@
         <v>11.01</v>
       </c>
       <c s="7" r="N99">
-        <v>148689529.8</v>
+        <v>148689529.80</v>
       </c>
       <c s="7" r="O99">
         <v>14037.91</v>
@@ -4757,7 +4757,7 @@
         </is>
       </c>
       <c s="6" r="D100">
-        <v>1195</v>
+        <v>1195.00</v>
       </c>
       <c s="7" r="E100">
         <v>6907349.14</v>
@@ -4787,7 +4787,7 @@
         <v>6.73</v>
       </c>
       <c s="7" r="N100">
-        <v>19233017.5</v>
+        <v>19233017.50</v>
       </c>
       <c s="7" r="O100">
         <v>16094.57</v>
@@ -4805,7 +4805,7 @@
         </is>
       </c>
       <c s="6" r="D101">
-        <v>4574</v>
+        <v>4574.00</v>
       </c>
       <c s="7" r="E101">
         <v>8833508.84</v>
@@ -4814,7 +4814,7 @@
         <v>1931.24</v>
       </c>
       <c s="7" r="G101">
-        <v>15.9</v>
+        <v>15.90</v>
       </c>
       <c s="7" r="H101">
         <v>43505178.38</v>
@@ -4838,7 +4838,7 @@
         <v>55539353.29</v>
       </c>
       <c s="7" r="O101">
-        <v>12142.4</v>
+        <v>12142.40</v>
       </c>
     </row>
     <row r="102" ht="14.4" customHeight="0">
@@ -4853,13 +4853,13 @@
         </is>
       </c>
       <c s="6" r="D102">
-        <v>10372</v>
+        <v>10372.00</v>
       </c>
       <c s="7" r="E102">
         <v>48272333.48</v>
       </c>
       <c s="7" r="F102">
-        <v>4654.1</v>
+        <v>4654.10</v>
       </c>
       <c s="7" r="G102">
         <v>31.38</v>
@@ -4880,13 +4880,13 @@
         <v>889.95</v>
       </c>
       <c s="7" r="M102">
-        <v>6</v>
+        <v>6.00</v>
       </c>
       <c s="7" r="N102">
-        <v>153826038.3</v>
+        <v>153826038.30</v>
       </c>
       <c s="7" r="O102">
-        <v>14830.9</v>
+        <v>14830.90</v>
       </c>
     </row>
     <row r="103" ht="14.4" customHeight="0">
@@ -4901,7 +4901,7 @@
         </is>
       </c>
       <c s="6" r="D103">
-        <v>3765</v>
+        <v>3765.00</v>
       </c>
       <c s="7" r="E103">
         <v>25329890.56</v>
@@ -4913,7 +4913,7 @@
         <v>44.58</v>
       </c>
       <c s="7" r="H103">
-        <v>28645929.4</v>
+        <v>28645929.40</v>
       </c>
       <c s="7" r="I103">
         <v>7608.48</v>
@@ -4928,13 +4928,13 @@
         <v>753.89</v>
       </c>
       <c s="7" r="M103">
-        <v>5</v>
+        <v>5.00</v>
       </c>
       <c s="7" r="N103">
         <v>56814231.79</v>
       </c>
       <c s="7" r="O103">
-        <v>15090.1</v>
+        <v>15090.10</v>
       </c>
     </row>
     <row r="104" ht="14.4" customHeight="0">
@@ -4949,7 +4949,7 @@
         </is>
       </c>
       <c s="6" r="D104">
-        <v>988</v>
+        <v>988.00</v>
       </c>
       <c s="7" r="E104">
         <v>8734684.39</v>
@@ -4964,7 +4964,7 @@
         <v>7525006.49</v>
       </c>
       <c s="7" r="I104">
-        <v>7616.4</v>
+        <v>7616.40</v>
       </c>
       <c s="7" r="J104">
         <v>41.63</v>
@@ -4997,7 +4997,7 @@
         </is>
       </c>
       <c s="6" r="D105">
-        <v>5084</v>
+        <v>5084.00</v>
       </c>
       <c s="7" r="E105">
         <v>24937944.89</v>
@@ -5045,7 +5045,7 @@
         </is>
       </c>
       <c s="6" r="D106">
-        <v>1262</v>
+        <v>1262.00</v>
       </c>
       <c s="7" r="E106">
         <v>3804400.54</v>
@@ -5093,7 +5093,7 @@
         </is>
       </c>
       <c s="6" r="D107">
-        <v>2985</v>
+        <v>2985.00</v>
       </c>
       <c s="7" r="E107">
         <v>15131438.49</v>
@@ -5111,7 +5111,7 @@
         <v>9549.26</v>
       </c>
       <c s="7" r="J107">
-        <v>60.5</v>
+        <v>60.50</v>
       </c>
       <c s="7" r="K107">
         <v>3481813.37</v>
@@ -5141,13 +5141,13 @@
         </is>
       </c>
       <c s="6" r="D108">
-        <v>1337</v>
+        <v>1337.00</v>
       </c>
       <c s="7" r="E108">
         <v>11003781.98</v>
       </c>
       <c s="7" r="F108">
-        <v>8230.2</v>
+        <v>8230.20</v>
       </c>
       <c s="7" r="G108">
         <v>50.13</v>
@@ -5156,7 +5156,7 @@
         <v>9539900.06</v>
       </c>
       <c s="7" r="I108">
-        <v>7135.3</v>
+        <v>7135.30</v>
       </c>
       <c s="7" r="J108">
         <v>43.46</v>
@@ -5189,7 +5189,7 @@
         </is>
       </c>
       <c s="6" r="D109">
-        <v>2154</v>
+        <v>2154.00</v>
       </c>
       <c s="7" r="E109">
         <v>15500687.14</v>
@@ -5207,7 +5207,7 @@
         <v>9909.11</v>
       </c>
       <c s="7" r="J109">
-        <v>49.6</v>
+        <v>49.60</v>
       </c>
       <c s="7" r="K109">
         <v>6187171.91</v>
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c s="6" r="D110">
-        <v>738</v>
+        <v>738.00</v>
       </c>
       <c s="7" r="E110">
         <v>4323396.25</v>
@@ -5255,7 +5255,7 @@
         <v>9683.32</v>
       </c>
       <c s="7" r="J110">
-        <v>58.2</v>
+        <v>58.20</v>
       </c>
       <c s="7" r="K110">
         <v>808366.37</v>
@@ -5267,7 +5267,7 @@
         <v>6.58</v>
       </c>
       <c s="7" r="N110">
-        <v>12278056.4</v>
+        <v>12278056.40</v>
       </c>
       <c s="7" r="O110">
         <v>16636.93</v>
@@ -5285,7 +5285,7 @@
         </is>
       </c>
       <c s="6" r="D111">
-        <v>1154</v>
+        <v>1154.00</v>
       </c>
       <c s="7" r="E111">
         <v>15817192.24</v>
@@ -5333,7 +5333,7 @@
         </is>
       </c>
       <c s="6" r="D112">
-        <v>4556</v>
+        <v>4556.00</v>
       </c>
       <c s="7" r="E112">
         <v>32399898.41</v>
@@ -5381,10 +5381,10 @@
         </is>
       </c>
       <c s="6" r="D113">
-        <v>864</v>
+        <v>864.00</v>
       </c>
       <c s="7" r="E113">
-        <v>4273203.3</v>
+        <v>4273203.30</v>
       </c>
       <c s="7" r="F113">
         <v>4945.84</v>
@@ -5402,7 +5402,7 @@
         <v>64.34</v>
       </c>
       <c s="7" r="K113">
-        <v>1124620.7</v>
+        <v>1124620.70</v>
       </c>
       <c s="7" r="L113">
         <v>1301.64</v>
@@ -5429,7 +5429,7 @@
         </is>
       </c>
       <c s="6" r="D114">
-        <v>3514</v>
+        <v>3514.00</v>
       </c>
       <c s="7" r="E114">
         <v>25105461.07</v>
@@ -5477,7 +5477,7 @@
         </is>
       </c>
       <c s="6" r="D115">
-        <v>6502</v>
+        <v>6502.00</v>
       </c>
       <c s="7" r="E115">
         <v>22442124.68</v>
@@ -5507,7 +5507,7 @@
         <v>5.43</v>
       </c>
       <c s="7" r="N115">
-        <v>82647124.7</v>
+        <v>82647124.70</v>
       </c>
       <c s="7" r="O115">
         <v>12711.03</v>
@@ -5525,7 +5525,7 @@
         </is>
       </c>
       <c s="6" r="D116">
-        <v>28835</v>
+        <v>28835.00</v>
       </c>
       <c s="7" r="E116">
         <v>155961890.72</v>
@@ -5573,7 +5573,7 @@
         </is>
       </c>
       <c s="6" r="D117">
-        <v>18402</v>
+        <v>18402.00</v>
       </c>
       <c s="7" r="E117">
         <v>100497735.07</v>
@@ -5621,10 +5621,10 @@
         </is>
       </c>
       <c s="6" r="D118">
-        <v>8539</v>
+        <v>8539.00</v>
       </c>
       <c s="7" r="E118">
-        <v>58807585.4</v>
+        <v>58807585.40</v>
       </c>
       <c s="7" r="F118">
         <v>6886.94</v>
@@ -5651,7 +5651,7 @@
         <v>2.34</v>
       </c>
       <c s="7" r="N118">
-        <v>124205603.6</v>
+        <v>124205603.60</v>
       </c>
       <c s="7" r="O118">
         <v>14545.69</v>
@@ -5669,19 +5669,19 @@
         </is>
       </c>
       <c s="6" r="D119">
-        <v>2287</v>
+        <v>2287.00</v>
       </c>
       <c s="7" r="E119">
         <v>12746143.74</v>
       </c>
       <c s="7" r="F119">
-        <v>5573.3</v>
+        <v>5573.30</v>
       </c>
       <c s="7" r="G119">
         <v>37.58</v>
       </c>
       <c s="7" r="H119">
-        <v>19357414.2</v>
+        <v>19357414.20</v>
       </c>
       <c s="7" r="I119">
         <v>8464.11</v>
@@ -5717,7 +5717,7 @@
         </is>
       </c>
       <c s="6" r="D120">
-        <v>31566</v>
+        <v>31566.00</v>
       </c>
       <c s="7" r="E120">
         <v>170499135.17</v>
@@ -5765,16 +5765,16 @@
         </is>
       </c>
       <c s="6" r="D121">
-        <v>3918</v>
+        <v>3918.00</v>
       </c>
       <c s="7" r="E121">
-        <v>17773273.4</v>
+        <v>17773273.40</v>
       </c>
       <c s="7" r="F121">
         <v>4536.31</v>
       </c>
       <c s="7" r="G121">
-        <v>32</v>
+        <v>32.00</v>
       </c>
       <c s="7" r="H121">
         <v>33625631.22</v>
@@ -5813,7 +5813,7 @@
         </is>
       </c>
       <c s="6" r="D122">
-        <v>3920</v>
+        <v>3920.00</v>
       </c>
       <c s="7" r="E122">
         <v>32193561.88</v>
@@ -5825,7 +5825,7 @@
         <v>50.89</v>
       </c>
       <c s="7" r="H122">
-        <v>28391194.9</v>
+        <v>28391194.90</v>
       </c>
       <c s="7" r="I122">
         <v>7242.65</v>
@@ -5861,10 +5861,10 @@
         </is>
       </c>
       <c s="6" r="D123">
-        <v>3565</v>
+        <v>3565.00</v>
       </c>
       <c s="7" r="E123">
-        <v>12356872.8</v>
+        <v>12356872.80</v>
       </c>
       <c s="7" r="F123">
         <v>3466.16</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c s="6" r="D124">
-        <v>3351</v>
+        <v>3351.00</v>
       </c>
       <c s="7" r="E124">
         <v>16232896.62</v>
@@ -5927,7 +5927,7 @@
         <v>8337.05</v>
       </c>
       <c s="7" r="J124">
-        <v>59</v>
+        <v>59.00</v>
       </c>
       <c s="7" r="K124">
         <v>3180666.47</v>
@@ -5957,7 +5957,7 @@
         </is>
       </c>
       <c s="6" r="D125">
-        <v>7611</v>
+        <v>7611.00</v>
       </c>
       <c s="7" r="E125">
         <v>26616705.94</v>
@@ -6005,7 +6005,7 @@
         </is>
       </c>
       <c s="6" r="D126">
-        <v>1250</v>
+        <v>1250.00</v>
       </c>
       <c s="7" r="E126">
         <v>5724581.94</v>
@@ -6053,10 +6053,10 @@
         </is>
       </c>
       <c s="6" r="D127">
-        <v>2842</v>
+        <v>2842.00</v>
       </c>
       <c s="7" r="E127">
-        <v>29103236.3</v>
+        <v>29103236.30</v>
       </c>
       <c s="7" r="F127">
         <v>10240.41</v>
@@ -6074,19 +6074,19 @@
         <v>32.83</v>
       </c>
       <c s="7" r="K127">
-        <v>6204929.8</v>
+        <v>6204929.80</v>
       </c>
       <c s="7" r="L127">
-        <v>2183.3</v>
+        <v>2183.30</v>
       </c>
       <c s="7" r="M127">
-        <v>11.8</v>
+        <v>11.80</v>
       </c>
       <c s="7" r="N127">
         <v>52566461.51</v>
       </c>
       <c s="7" r="O127">
-        <v>18496.3</v>
+        <v>18496.30</v>
       </c>
     </row>
     <row r="128" ht="14.4" customHeight="0">
@@ -6101,10 +6101,10 @@
         </is>
       </c>
       <c s="6" r="D128">
-        <v>288</v>
+        <v>288.00</v>
       </c>
       <c s="7" r="E128">
-        <v>1779450</v>
+        <v>1779450.00</v>
       </c>
       <c s="7" r="F128">
         <v>6178.65</v>
@@ -6131,7 +6131,7 @@
         <v>15.72</v>
       </c>
       <c s="7" r="N128">
-        <v>7138443.2</v>
+        <v>7138443.20</v>
       </c>
       <c s="7" r="O128">
         <v>24786.26</v>
@@ -6149,7 +6149,7 @@
         </is>
       </c>
       <c s="6" r="D129">
-        <v>2182</v>
+        <v>2182.00</v>
       </c>
       <c s="7" r="E129">
         <v>27334211.07</v>
@@ -6158,7 +6158,7 @@
         <v>12527.14</v>
       </c>
       <c s="7" r="G129">
-        <v>66.1</v>
+        <v>66.10</v>
       </c>
       <c s="7" r="H129">
         <v>11838038.64</v>
@@ -6182,7 +6182,7 @@
         <v>41349762.94</v>
       </c>
       <c s="7" r="O129">
-        <v>18950.4</v>
+        <v>18950.40</v>
       </c>
     </row>
     <row r="130" ht="14.4" customHeight="0">
@@ -6197,7 +6197,7 @@
         </is>
       </c>
       <c s="6" r="D130">
-        <v>556</v>
+        <v>556.00</v>
       </c>
       <c s="7" r="E130">
         <v>4486186.47</v>
@@ -6212,7 +6212,7 @@
         <v>5659746.14</v>
       </c>
       <c s="7" r="I130">
-        <v>10179.4</v>
+        <v>10179.40</v>
       </c>
       <c s="7" r="J130">
         <v>48.93</v>
@@ -6245,7 +6245,7 @@
         </is>
       </c>
       <c s="6" r="D131">
-        <v>28048</v>
+        <v>28048.00</v>
       </c>
       <c s="7" r="E131">
         <v>151006003.97</v>
@@ -6293,10 +6293,10 @@
         </is>
       </c>
       <c s="6" r="D132">
-        <v>15298</v>
+        <v>15298.00</v>
       </c>
       <c s="7" r="E132">
-        <v>108506456.6</v>
+        <v>108506456.60</v>
       </c>
       <c s="7" r="F132">
         <v>7092.85</v>
@@ -6323,7 +6323,7 @@
         <v>7.32</v>
       </c>
       <c s="7" r="N132">
-        <v>241700206.9</v>
+        <v>241700206.90</v>
       </c>
       <c s="7" r="O132">
         <v>15799.46</v>
@@ -6341,7 +6341,7 @@
         </is>
       </c>
       <c s="6" r="D133">
-        <v>1183</v>
+        <v>1183.00</v>
       </c>
       <c s="7" r="E133">
         <v>3285965.58</v>
@@ -6389,7 +6389,7 @@
         </is>
       </c>
       <c s="6" r="D134">
-        <v>1990</v>
+        <v>1990.00</v>
       </c>
       <c s="7" r="E134">
         <v>9194150.21</v>
@@ -6404,7 +6404,7 @@
         <v>17250919.88</v>
       </c>
       <c s="7" r="I134">
-        <v>8668.8</v>
+        <v>8668.80</v>
       </c>
       <c s="7" r="J134">
         <v>59.43</v>
@@ -6416,7 +6416,7 @@
         <v>1297.76</v>
       </c>
       <c s="7" r="M134">
-        <v>8.9</v>
+        <v>8.90</v>
       </c>
       <c s="7" r="N134">
         <v>29027604.71</v>
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c s="6" r="D135">
-        <v>1287</v>
+        <v>1287.00</v>
       </c>
       <c s="7" r="E135">
         <v>6759307.08</v>
@@ -6485,13 +6485,13 @@
         </is>
       </c>
       <c s="6" r="D136">
-        <v>8974</v>
+        <v>8974.00</v>
       </c>
       <c s="7" r="E136">
-        <v>49736569.2</v>
+        <v>49736569.20</v>
       </c>
       <c s="7" r="F136">
-        <v>5542.3</v>
+        <v>5542.30</v>
       </c>
       <c s="7" r="G136">
         <v>37.32</v>
@@ -6533,7 +6533,7 @@
         </is>
       </c>
       <c s="6" r="D137">
-        <v>3705</v>
+        <v>3705.00</v>
       </c>
       <c s="7" r="E137">
         <v>14989120.62</v>
@@ -6557,7 +6557,7 @@
         <v>2926961.53</v>
       </c>
       <c s="7" r="L137">
-        <v>790</v>
+        <v>790.00</v>
       </c>
       <c s="7" r="M137">
         <v>5.82</v>
@@ -6566,7 +6566,7 @@
         <v>50312418.46</v>
       </c>
       <c s="7" r="O137">
-        <v>13579.6</v>
+        <v>13579.60</v>
       </c>
     </row>
     <row r="138" ht="14.4" customHeight="0">
@@ -6581,7 +6581,7 @@
         </is>
       </c>
       <c s="6" r="D138">
-        <v>320</v>
+        <v>320.00</v>
       </c>
       <c s="7" r="E138">
         <v>3179430.19</v>
@@ -6596,7 +6596,7 @@
         <v>3751006.53</v>
       </c>
       <c s="7" r="I138">
-        <v>11721.9</v>
+        <v>11721.90</v>
       </c>
       <c s="7" r="J138">
         <v>41.86</v>
@@ -6629,19 +6629,19 @@
         </is>
       </c>
       <c s="6" r="D139">
-        <v>3442</v>
+        <v>3442.00</v>
       </c>
       <c s="7" r="E139">
         <v>16640701.26</v>
       </c>
       <c s="7" r="F139">
-        <v>4834.6</v>
+        <v>4834.60</v>
       </c>
       <c s="7" r="G139">
         <v>26.12</v>
       </c>
       <c s="7" r="H139">
-        <v>29863958.7</v>
+        <v>29863958.70</v>
       </c>
       <c s="7" r="I139">
         <v>8676.34</v>
@@ -6677,7 +6677,7 @@
         </is>
       </c>
       <c s="6" r="D140">
-        <v>349</v>
+        <v>349.00</v>
       </c>
       <c s="7" r="E140">
         <v>4610704.59</v>
@@ -6704,7 +6704,7 @@
         <v>5951.36</v>
       </c>
       <c s="7" r="M140">
-        <v>20.5</v>
+        <v>20.50</v>
       </c>
       <c s="7" r="N140">
         <v>10130852.56</v>
@@ -6725,10 +6725,10 @@
         </is>
       </c>
       <c s="6" r="D141">
-        <v>184</v>
+        <v>184.00</v>
       </c>
       <c s="7" r="E141">
-        <v>1569039.6</v>
+        <v>1569039.60</v>
       </c>
       <c s="7" r="F141">
         <v>8527.39</v>
@@ -6737,13 +6737,13 @@
         <v>29.04</v>
       </c>
       <c s="7" r="H141">
-        <v>3100589.9</v>
+        <v>3100589.90</v>
       </c>
       <c s="7" r="I141">
         <v>16851.03</v>
       </c>
       <c s="7" r="J141">
-        <v>57.4</v>
+        <v>57.40</v>
       </c>
       <c s="7" r="K141">
         <v>732470.13</v>
@@ -6773,7 +6773,7 @@
         </is>
       </c>
       <c s="6" r="D142">
-        <v>3374</v>
+        <v>3374.00</v>
       </c>
       <c s="7" r="E142">
         <v>10073242.48</v>
@@ -6806,7 +6806,7 @@
         <v>49260082.21</v>
       </c>
       <c s="7" r="O142">
-        <v>14599.9</v>
+        <v>14599.90</v>
       </c>
     </row>
     <row r="143" ht="14.4" customHeight="0">
@@ -6821,13 +6821,13 @@
         </is>
       </c>
       <c s="6" r="D143">
-        <v>1131</v>
+        <v>1131.00</v>
       </c>
       <c s="7" r="E143">
         <v>5790723.96</v>
       </c>
       <c s="7" r="F143">
-        <v>5120</v>
+        <v>5120.00</v>
       </c>
       <c s="7" r="G143">
         <v>28.56</v>
@@ -6869,13 +6869,13 @@
         </is>
       </c>
       <c s="6" r="D144">
-        <v>1448</v>
+        <v>1448.00</v>
       </c>
       <c s="7" r="E144">
         <v>5466781.68</v>
       </c>
       <c s="7" r="F144">
-        <v>3775.4</v>
+        <v>3775.40</v>
       </c>
       <c s="7" r="G144">
         <v>24.49</v>
@@ -6917,7 +6917,7 @@
         </is>
       </c>
       <c s="6" r="D145">
-        <v>896</v>
+        <v>896.00</v>
       </c>
       <c s="7" r="E145">
         <v>6736600.32</v>
@@ -6947,7 +6947,7 @@
         <v>24.44</v>
       </c>
       <c s="7" r="N145">
-        <v>19397835.1</v>
+        <v>19397835.10</v>
       </c>
       <c s="7" r="O145">
         <v>21649.37</v>
@@ -6965,10 +6965,10 @@
         </is>
       </c>
       <c s="6" r="D146">
-        <v>5534</v>
+        <v>5534.00</v>
       </c>
       <c s="7" r="E146">
-        <v>22045658.7</v>
+        <v>22045658.70</v>
       </c>
       <c s="7" r="F146">
         <v>3983.68</v>
@@ -7013,7 +7013,7 @@
         </is>
       </c>
       <c s="6" r="D147">
-        <v>7297</v>
+        <v>7297.00</v>
       </c>
       <c s="7" r="E147">
         <v>28697857.13</v>
@@ -7061,7 +7061,7 @@
         </is>
       </c>
       <c s="6" r="D148">
-        <v>3002</v>
+        <v>3002.00</v>
       </c>
       <c s="7" r="E148">
         <v>11416813.25</v>
@@ -7073,7 +7073,7 @@
         <v>25.43</v>
       </c>
       <c s="7" r="H148">
-        <v>29380531.2</v>
+        <v>29380531.20</v>
       </c>
       <c s="7" r="I148">
         <v>9786.99</v>
@@ -7091,7 +7091,7 @@
         <v>9.14</v>
       </c>
       <c s="7" r="N148">
-        <v>44902563.7</v>
+        <v>44902563.70</v>
       </c>
       <c s="7" r="O148">
         <v>14957.55</v>
@@ -7109,13 +7109,13 @@
         </is>
       </c>
       <c s="6" r="D149">
-        <v>920</v>
+        <v>920.00</v>
       </c>
       <c s="7" r="E149">
         <v>12370136.42</v>
       </c>
       <c s="7" r="F149">
-        <v>13445.8</v>
+        <v>13445.80</v>
       </c>
       <c s="7" r="G149">
         <v>66.43</v>
@@ -7136,7 +7136,7 @@
         <v>709.36</v>
       </c>
       <c s="7" r="M149">
-        <v>3.5</v>
+        <v>3.50</v>
       </c>
       <c s="7" r="N149">
         <v>18621502.82</v>
@@ -7157,7 +7157,7 @@
         </is>
       </c>
       <c s="6" r="D150">
-        <v>963</v>
+        <v>963.00</v>
       </c>
       <c s="7" r="E150">
         <v>3756001.27</v>
@@ -7205,13 +7205,13 @@
         </is>
       </c>
       <c s="6" r="D151">
-        <v>11939</v>
+        <v>11939.00</v>
       </c>
       <c s="7" r="E151">
         <v>73143130.25</v>
       </c>
       <c s="7" r="F151">
-        <v>6126.4</v>
+        <v>6126.40</v>
       </c>
       <c s="7" r="G151">
         <v>39.56</v>
@@ -7235,7 +7235,7 @@
         <v>8.45</v>
       </c>
       <c s="7" r="N151">
-        <v>184877252</v>
+        <v>184877252.00</v>
       </c>
       <c s="7" r="O151">
         <v>15485.15</v>
@@ -7253,7 +7253,7 @@
         </is>
       </c>
       <c s="6" r="D152">
-        <v>1054</v>
+        <v>1054.00</v>
       </c>
       <c s="7" r="E152">
         <v>4654680.94</v>
@@ -7262,10 +7262,10 @@
         <v>4416.21</v>
       </c>
       <c s="7" r="G152">
-        <v>24.7</v>
+        <v>24.70</v>
       </c>
       <c s="7" r="H152">
-        <v>11197606.4</v>
+        <v>11197606.40</v>
       </c>
       <c s="7" r="I152">
         <v>10623.91</v>
@@ -7286,7 +7286,7 @@
         <v>18842147.87</v>
       </c>
       <c s="7" r="O152">
-        <v>17876.8</v>
+        <v>17876.80</v>
       </c>
     </row>
     <row r="153" ht="14.4" customHeight="0">
@@ -7301,7 +7301,7 @@
         </is>
       </c>
       <c s="6" r="D153">
-        <v>702</v>
+        <v>702.00</v>
       </c>
       <c s="7" r="E153">
         <v>6639673.98</v>
@@ -7349,7 +7349,7 @@
         </is>
       </c>
       <c s="6" r="D154">
-        <v>2905</v>
+        <v>2905.00</v>
       </c>
       <c s="7" r="E154">
         <v>25355391.89</v>
@@ -7364,7 +7364,7 @@
         <v>20984546.08</v>
       </c>
       <c s="7" r="I154">
-        <v>7223.6</v>
+        <v>7223.60</v>
       </c>
       <c s="7" r="J154">
         <v>42.34</v>
@@ -7397,10 +7397,10 @@
         </is>
       </c>
       <c s="6" r="D155">
-        <v>3885</v>
+        <v>3885.00</v>
       </c>
       <c s="7" r="E155">
-        <v>16181630.9</v>
+        <v>16181630.90</v>
       </c>
       <c s="7" r="F155">
         <v>4165.16</v>
@@ -7445,10 +7445,10 @@
         </is>
       </c>
       <c s="6" r="D156">
-        <v>8103</v>
+        <v>8103.00</v>
       </c>
       <c s="7" r="E156">
-        <v>43900587.9</v>
+        <v>43900587.90</v>
       </c>
       <c s="7" r="F156">
         <v>5417.82</v>
@@ -7493,7 +7493,7 @@
         </is>
       </c>
       <c s="6" r="D157">
-        <v>14556</v>
+        <v>14556.00</v>
       </c>
       <c s="7" r="E157">
         <v>90950994.62</v>
@@ -7541,7 +7541,7 @@
         </is>
       </c>
       <c s="6" r="D158">
-        <v>5673</v>
+        <v>5673.00</v>
       </c>
       <c s="7" r="E158">
         <v>20589472.65</v>
@@ -7550,7 +7550,7 @@
         <v>3629.38</v>
       </c>
       <c s="7" r="G158">
-        <v>23.2</v>
+        <v>23.20</v>
       </c>
       <c s="7" r="H158">
         <v>60484271.04</v>
@@ -7565,7 +7565,7 @@
         <v>7659691.86</v>
       </c>
       <c s="7" r="L158">
-        <v>1350.2</v>
+        <v>1350.20</v>
       </c>
       <c s="7" r="M158">
         <v>8.63</v>
@@ -7589,7 +7589,7 @@
         </is>
       </c>
       <c s="6" r="D159">
-        <v>662</v>
+        <v>662.00</v>
       </c>
       <c s="7" r="E159">
         <v>4514028.96</v>
@@ -7601,7 +7601,7 @@
         <v>35.65</v>
       </c>
       <c s="7" r="H159">
-        <v>7073638.2</v>
+        <v>7073638.20</v>
       </c>
       <c s="7" r="I159">
         <v>10685.25</v>
@@ -7637,7 +7637,7 @@
         </is>
       </c>
       <c s="6" r="D160">
-        <v>2610</v>
+        <v>2610.00</v>
       </c>
       <c s="7" r="E160">
         <v>14800611.24</v>
@@ -7670,7 +7670,7 @@
         <v>38880661.87</v>
       </c>
       <c s="7" r="O160">
-        <v>14896.8</v>
+        <v>14896.80</v>
       </c>
     </row>
     <row r="161" ht="14.4" customHeight="0">
@@ -7685,19 +7685,19 @@
         </is>
       </c>
       <c s="6" r="D161">
-        <v>5159</v>
+        <v>5159.00</v>
       </c>
       <c s="7" r="E161">
         <v>17718584.75</v>
       </c>
       <c s="7" r="F161">
-        <v>3434.5</v>
+        <v>3434.50</v>
       </c>
       <c s="7" r="G161">
         <v>24.61</v>
       </c>
       <c s="7" r="H161">
-        <v>47404358.2</v>
+        <v>47404358.20</v>
       </c>
       <c s="7" r="I161">
         <v>9188.67</v>
@@ -7733,7 +7733,7 @@
         </is>
       </c>
       <c s="6" r="D162">
-        <v>216</v>
+        <v>216.00</v>
       </c>
       <c s="7" r="E162">
         <v>1967844.22</v>
@@ -7745,7 +7745,7 @@
         <v>35.14</v>
       </c>
       <c s="7" r="H162">
-        <v>3183156</v>
+        <v>3183156.00</v>
       </c>
       <c s="7" r="I162">
         <v>14736.83</v>
@@ -7754,7 +7754,7 @@
         <v>56.83</v>
       </c>
       <c s="7" r="K162">
-        <v>449763.4</v>
+        <v>449763.40</v>
       </c>
       <c s="7" r="L162">
         <v>2082.24</v>
@@ -7781,7 +7781,7 @@
         </is>
       </c>
       <c s="6" r="D163">
-        <v>788</v>
+        <v>788.00</v>
       </c>
       <c s="7" r="E163">
         <v>3226919.67</v>
@@ -7793,7 +7793,7 @@
         <v>23.83</v>
       </c>
       <c s="7" r="H163">
-        <v>8977235.7</v>
+        <v>8977235.70</v>
       </c>
       <c s="7" r="I163">
         <v>11392.43</v>
@@ -7829,10 +7829,10 @@
         </is>
       </c>
       <c s="6" r="D164">
-        <v>3707</v>
+        <v>3707.00</v>
       </c>
       <c s="7" r="E164">
-        <v>23892509.3</v>
+        <v>23892509.30</v>
       </c>
       <c s="7" r="F164">
         <v>6445.24</v>
@@ -7877,7 +7877,7 @@
         </is>
       </c>
       <c s="6" r="D165">
-        <v>12078</v>
+        <v>12078.00</v>
       </c>
       <c s="7" r="E165">
         <v>45710168.27</v>
@@ -7925,7 +7925,7 @@
         </is>
       </c>
       <c s="6" r="D166">
-        <v>1070</v>
+        <v>1070.00</v>
       </c>
       <c s="7" r="E166">
         <v>4113637.52</v>
@@ -7940,10 +7940,10 @@
         <v>11034160.99</v>
       </c>
       <c s="7" r="I166">
-        <v>10312.3</v>
+        <v>10312.30</v>
       </c>
       <c s="7" r="J166">
-        <v>64.8</v>
+        <v>64.80</v>
       </c>
       <c s="7" r="K166">
         <v>1879519.26</v>
@@ -7973,7 +7973,7 @@
         </is>
       </c>
       <c s="6" r="D167">
-        <v>1211</v>
+        <v>1211.00</v>
       </c>
       <c s="7" r="E167">
         <v>8971772.12</v>
@@ -7988,7 +7988,7 @@
         <v>10066194.44</v>
       </c>
       <c s="7" r="I167">
-        <v>8312.3</v>
+        <v>8312.30</v>
       </c>
       <c s="7" r="J167">
         <v>48.63</v>
@@ -8021,7 +8021,7 @@
         </is>
       </c>
       <c s="6" r="D168">
-        <v>990</v>
+        <v>990.00</v>
       </c>
       <c s="7" r="E168">
         <v>8286130.21</v>
@@ -8042,7 +8042,7 @@
         <v>46.83</v>
       </c>
       <c s="7" r="K168">
-        <v>1116392.9</v>
+        <v>1116392.90</v>
       </c>
       <c s="7" r="L168">
         <v>1127.67</v>
@@ -8069,7 +8069,7 @@
         </is>
       </c>
       <c s="6" r="D169">
-        <v>2937</v>
+        <v>2937.00</v>
       </c>
       <c s="7" r="E169">
         <v>10234137.15</v>
@@ -8081,13 +8081,13 @@
         <v>24.92</v>
       </c>
       <c s="7" r="H169">
-        <v>26450622.8</v>
+        <v>26450622.80</v>
       </c>
       <c s="7" r="I169">
-        <v>9006</v>
+        <v>9006.00</v>
       </c>
       <c s="7" r="J169">
-        <v>64.4</v>
+        <v>64.40</v>
       </c>
       <c s="7" r="K169">
         <v>4385901.76</v>
@@ -8117,7 +8117,7 @@
         </is>
       </c>
       <c s="6" r="D170">
-        <v>49515</v>
+        <v>49515.00</v>
       </c>
       <c s="7" r="E170">
         <v>980019806.77</v>
@@ -8165,7 +8165,7 @@
         </is>
       </c>
       <c s="6" r="D171">
-        <v>2278</v>
+        <v>2278.00</v>
       </c>
       <c s="7" r="E171">
         <v>8197721.61</v>
@@ -8192,7 +8192,7 @@
         <v>487.55</v>
       </c>
       <c s="7" r="M171">
-        <v>3.7</v>
+        <v>3.70</v>
       </c>
       <c s="7" r="N171">
         <v>30008492.39</v>
@@ -8213,7 +8213,7 @@
         </is>
       </c>
       <c s="6" r="D172">
-        <v>6129</v>
+        <v>6129.00</v>
       </c>
       <c s="7" r="E172">
         <v>53650277.12</v>
@@ -8222,7 +8222,7 @@
         <v>8753.51</v>
       </c>
       <c s="7" r="G172">
-        <v>57.3</v>
+        <v>57.30</v>
       </c>
       <c s="7" r="H172">
         <v>37785744.47</v>
@@ -8261,7 +8261,7 @@
         </is>
       </c>
       <c s="6" r="D173">
-        <v>4188</v>
+        <v>4188.00</v>
       </c>
       <c s="7" r="E173">
         <v>18527614.56</v>
@@ -8288,7 +8288,7 @@
         <v>708.04</v>
       </c>
       <c s="7" r="M173">
-        <v>5.9</v>
+        <v>5.90</v>
       </c>
       <c s="7" r="N173">
         <v>50249463.56</v>
@@ -8309,7 +8309,7 @@
         </is>
       </c>
       <c s="6" r="D174">
-        <v>5803</v>
+        <v>5803.00</v>
       </c>
       <c s="7" r="E174">
         <v>27587333.64</v>
@@ -8357,7 +8357,7 @@
         </is>
       </c>
       <c s="6" r="D175">
-        <v>4682</v>
+        <v>4682.00</v>
       </c>
       <c s="7" r="E175">
         <v>34268085.27</v>
@@ -8390,7 +8390,7 @@
         <v>68229411.73</v>
       </c>
       <c s="7" r="O175">
-        <v>14572.7</v>
+        <v>14572.70</v>
       </c>
     </row>
     <row r="176" ht="14.4" customHeight="0">
@@ -8405,7 +8405,7 @@
         </is>
       </c>
       <c s="6" r="D176">
-        <v>1268</v>
+        <v>1268.00</v>
       </c>
       <c s="7" r="E176">
         <v>4170641.75</v>
@@ -8417,7 +8417,7 @@
         <v>24.87</v>
       </c>
       <c s="7" r="H176">
-        <v>11951262.2</v>
+        <v>11951262.20</v>
       </c>
       <c s="7" r="I176">
         <v>9425.29</v>
@@ -8453,7 +8453,7 @@
         </is>
       </c>
       <c s="6" r="D177">
-        <v>1884</v>
+        <v>1884.00</v>
       </c>
       <c s="7" r="E177">
         <v>18925673.95</v>
@@ -8468,7 +8468,7 @@
         <v>14666372.72</v>
       </c>
       <c s="7" r="I177">
-        <v>7784.7</v>
+        <v>7784.70</v>
       </c>
       <c s="7" r="J177">
         <v>42.41</v>
@@ -8501,13 +8501,13 @@
         </is>
       </c>
       <c s="6" r="D178">
-        <v>7780</v>
+        <v>7780.00</v>
       </c>
       <c s="7" r="E178">
         <v>45143450.44</v>
       </c>
       <c s="7" r="F178">
-        <v>5802.5</v>
+        <v>5802.50</v>
       </c>
       <c s="7" r="G178">
         <v>38.79</v>
@@ -8549,22 +8549,22 @@
         </is>
       </c>
       <c s="6" r="D179">
-        <v>5302</v>
+        <v>5302.00</v>
       </c>
       <c s="7" r="E179">
         <v>67201275.85</v>
       </c>
       <c s="7" r="F179">
-        <v>12674.7</v>
+        <v>12674.70</v>
       </c>
       <c s="7" r="G179">
-        <v>60.8</v>
+        <v>60.80</v>
       </c>
       <c s="7" r="H179">
         <v>41162080.05</v>
       </c>
       <c s="7" r="I179">
-        <v>7763.5</v>
+        <v>7763.50</v>
       </c>
       <c s="7" r="J179">
         <v>37.24</v>
@@ -8597,13 +8597,13 @@
         </is>
       </c>
       <c s="6" r="D180">
-        <v>2244</v>
+        <v>2244.00</v>
       </c>
       <c s="7" r="E180">
         <v>14839788.18</v>
       </c>
       <c s="7" r="F180">
-        <v>6613.1</v>
+        <v>6613.10</v>
       </c>
       <c s="7" r="G180">
         <v>42.84</v>
@@ -8645,7 +8645,7 @@
         </is>
       </c>
       <c s="6" r="D181">
-        <v>9024</v>
+        <v>9024.00</v>
       </c>
       <c s="7" r="E181">
         <v>52964653.35</v>
@@ -8675,7 +8675,7 @@
         <v>5.83</v>
       </c>
       <c s="7" r="N181">
-        <v>116035835.9</v>
+        <v>116035835.90</v>
       </c>
       <c s="7" r="O181">
         <v>12858.58</v>
@@ -8693,10 +8693,10 @@
         </is>
       </c>
       <c s="6" r="D182">
-        <v>4161</v>
+        <v>4161.00</v>
       </c>
       <c s="7" r="E182">
-        <v>21265925.8</v>
+        <v>21265925.80</v>
       </c>
       <c s="7" r="F182">
         <v>5110.77</v>
@@ -8705,7 +8705,7 @@
         <v>41.36</v>
       </c>
       <c s="7" r="H182">
-        <v>28801265.4</v>
+        <v>28801265.40</v>
       </c>
       <c s="7" r="I182">
         <v>6921.72</v>
@@ -8741,13 +8741,13 @@
         </is>
       </c>
       <c s="6" r="D183">
-        <v>9108</v>
+        <v>9108.00</v>
       </c>
       <c s="7" r="E183">
         <v>93617478.84</v>
       </c>
       <c s="7" r="F183">
-        <v>10278.6</v>
+        <v>10278.60</v>
       </c>
       <c s="7" r="G183">
         <v>55.39</v>
@@ -8789,7 +8789,7 @@
         </is>
       </c>
       <c s="6" r="D184">
-        <v>1602</v>
+        <v>1602.00</v>
       </c>
       <c s="7" r="E184">
         <v>2549829.54</v>
@@ -8837,7 +8837,7 @@
         </is>
       </c>
       <c s="6" r="D185">
-        <v>360</v>
+        <v>360.00</v>
       </c>
       <c s="7" r="E185">
         <v>25830.61</v>
@@ -8849,10 +8849,10 @@
         <v>0.24</v>
       </c>
       <c s="7" r="H185">
-        <v>5507675</v>
+        <v>5507675.00</v>
       </c>
       <c s="7" r="I185">
-        <v>15299.1</v>
+        <v>15299.10</v>
       </c>
       <c s="7" r="J185">
         <v>51.97</v>
@@ -8867,7 +8867,7 @@
         <v>47.79</v>
       </c>
       <c s="7" r="N185">
-        <v>10598379</v>
+        <v>10598379.00</v>
       </c>
       <c s="7" r="O185">
         <v>29439.94</v>
@@ -8885,7 +8885,7 @@
         </is>
       </c>
       <c s="6" r="D186">
-        <v>10151</v>
+        <v>10151.00</v>
       </c>
       <c s="7" r="E186">
         <v>191698.66</v>
@@ -8912,7 +8912,7 @@
         <v>1100.28</v>
       </c>
       <c s="7" r="M186">
-        <v>9.4</v>
+        <v>9.40</v>
       </c>
       <c s="7" r="N186">
         <v>118874676.26</v>
@@ -8933,7 +8933,7 @@
         </is>
       </c>
       <c s="6" r="D187">
-        <v>7008</v>
+        <v>7008.00</v>
       </c>
       <c s="8" t="str" r="E187"/>
       <c s="8" t="str" r="F187"/>
@@ -8957,7 +8957,7 @@
         <v>5.71</v>
       </c>
       <c s="7" r="N187">
-        <v>71469465</v>
+        <v>71469465.00</v>
       </c>
       <c s="7" r="O187">
         <v>10198.26</v>
@@ -8975,7 +8975,7 @@
         </is>
       </c>
       <c s="6" r="D188">
-        <v>431</v>
+        <v>431.00</v>
       </c>
       <c s="7" r="E188">
         <v>534946.83</v>
@@ -8987,13 +8987,13 @@
         <v>7.15</v>
       </c>
       <c s="7" r="H188">
-        <v>6461115</v>
+        <v>6461115.00</v>
       </c>
       <c s="7" r="I188">
         <v>14990.99</v>
       </c>
       <c s="7" r="J188">
-        <v>86.3</v>
+        <v>86.30</v>
       </c>
       <c s="7" r="K188">
         <v>490447.25</v>
@@ -9008,7 +9008,7 @@
         <v>7486509.08</v>
       </c>
       <c s="7" r="O188">
-        <v>17370.1</v>
+        <v>17370.10</v>
       </c>
     </row>
     <row r="189" ht="14.4" customHeight="0">
@@ -9023,7 +9023,7 @@
         </is>
       </c>
       <c s="6" r="D189">
-        <v>1382</v>
+        <v>1382.00</v>
       </c>
       <c s="7" r="E189">
         <v>3304170.73</v>
@@ -9035,10 +9035,10 @@
         <v>15.13</v>
       </c>
       <c s="7" r="H189">
-        <v>16808296</v>
+        <v>16808296.00</v>
       </c>
       <c s="7" r="I189">
-        <v>12162.3</v>
+        <v>12162.30</v>
       </c>
       <c s="7" r="J189">
         <v>76.96</v>
@@ -9071,7 +9071,7 @@
         </is>
       </c>
       <c s="6" r="D190">
-        <v>849</v>
+        <v>849.00</v>
       </c>
       <c s="7" r="E190">
         <v>7829834.33</v>
@@ -9104,7 +9104,7 @@
         <v>12084755.03</v>
       </c>
       <c s="7" r="O190">
-        <v>14234.1</v>
+        <v>14234.10</v>
       </c>
     </row>
     <row r="191" ht="14.4" customHeight="0">
@@ -9119,7 +9119,7 @@
         </is>
       </c>
       <c s="6" r="D191">
-        <v>949</v>
+        <v>949.00</v>
       </c>
       <c s="7" r="E191">
         <v>16632.11</v>
@@ -9134,7 +9134,7 @@
         <v>12161912.72</v>
       </c>
       <c s="7" r="I191">
-        <v>12815.5</v>
+        <v>12815.50</v>
       </c>
       <c s="7" r="J191">
         <v>90.63</v>
@@ -9167,7 +9167,7 @@
         </is>
       </c>
       <c s="6" r="D192">
-        <v>1009</v>
+        <v>1009.00</v>
       </c>
       <c s="7" r="E192">
         <v>102038.44</v>
@@ -9188,7 +9188,7 @@
         <v>97.62</v>
       </c>
       <c s="7" r="K192">
-        <v>216108</v>
+        <v>216108.00</v>
       </c>
       <c s="7" r="L192">
         <v>214.18</v>
@@ -9215,7 +9215,7 @@
         </is>
       </c>
       <c s="6" r="D193">
-        <v>1328</v>
+        <v>1328.00</v>
       </c>
       <c s="7" r="E193">
         <v>69681.78</v>
@@ -9227,7 +9227,7 @@
         <v>0.33</v>
       </c>
       <c s="7" r="H193">
-        <v>19606536.1</v>
+        <v>19606536.10</v>
       </c>
       <c s="7" r="I193">
         <v>14763.96</v>
@@ -9263,7 +9263,7 @@
         </is>
       </c>
       <c s="6" r="D194">
-        <v>1066</v>
+        <v>1066.00</v>
       </c>
       <c s="7" r="E194">
         <v>819018.93</v>
@@ -9311,19 +9311,19 @@
         </is>
       </c>
       <c s="6" r="D195">
-        <v>150</v>
+        <v>150.00</v>
       </c>
       <c s="7" r="E195">
-        <v>399719.9</v>
+        <v>399719.90</v>
       </c>
       <c s="7" r="F195">
-        <v>2664.8</v>
+        <v>2664.80</v>
       </c>
       <c s="7" r="G195">
         <v>15.21</v>
       </c>
       <c s="7" r="H195">
-        <v>2206205</v>
+        <v>2206205.00</v>
       </c>
       <c s="7" r="I195">
         <v>14708.03</v>
@@ -9359,7 +9359,7 @@
         </is>
       </c>
       <c s="6" r="D196">
-        <v>140</v>
+        <v>140.00</v>
       </c>
       <c s="7" r="E196">
         <v>2666960.37</v>
@@ -9371,7 +9371,7 @@
         <v>70.06</v>
       </c>
       <c s="7" r="H196">
-        <v>1097759</v>
+        <v>1097759.00</v>
       </c>
       <c s="7" r="I196">
         <v>7841.14</v>
@@ -9386,7 +9386,7 @@
         <v>299.69</v>
       </c>
       <c s="7" r="M196">
-        <v>1.1</v>
+        <v>1.10</v>
       </c>
       <c s="7" r="N196">
         <v>3806675.83</v>
@@ -9407,10 +9407,10 @@
         </is>
       </c>
       <c s="6" r="D197">
-        <v>202</v>
+        <v>202.00</v>
       </c>
       <c s="7" r="E197">
-        <v>271368</v>
+        <v>271368.00</v>
       </c>
       <c s="7" r="F197">
         <v>1343.41</v>
@@ -9419,7 +9419,7 @@
         <v>8.29</v>
       </c>
       <c s="7" r="H197">
-        <v>2725880</v>
+        <v>2725880.00</v>
       </c>
       <c s="7" r="I197">
         <v>13494.46</v>
@@ -9428,7 +9428,7 @@
         <v>83.26</v>
       </c>
       <c s="7" r="K197">
-        <v>276576</v>
+        <v>276576.00</v>
       </c>
       <c s="7" r="L197">
         <v>1369.19</v>
@@ -9437,7 +9437,7 @@
         <v>8.45</v>
       </c>
       <c s="7" r="N197">
-        <v>3273824</v>
+        <v>3273824.00</v>
       </c>
       <c s="7" r="O197">
         <v>16207.06</v>
@@ -9455,7 +9455,7 @@
         </is>
       </c>
       <c s="6" r="D198">
-        <v>584</v>
+        <v>584.00</v>
       </c>
       <c s="7" r="E198">
         <v>56451.61</v>
@@ -9467,7 +9467,7 @@
         <v>0.63</v>
       </c>
       <c s="7" r="H198">
-        <v>8335974</v>
+        <v>8335974.00</v>
       </c>
       <c s="7" r="I198">
         <v>14273.93</v>
@@ -9503,7 +9503,7 @@
         </is>
       </c>
       <c s="6" r="D199">
-        <v>646</v>
+        <v>646.00</v>
       </c>
       <c s="8" t="str" r="E199"/>
       <c s="8" t="str" r="F199"/>
@@ -9545,7 +9545,7 @@
         </is>
       </c>
       <c s="6" r="D200">
-        <v>459</v>
+        <v>459.00</v>
       </c>
       <c s="7" r="E200">
         <v>617347.27</v>
@@ -9557,7 +9557,7 @@
         <v>5.72</v>
       </c>
       <c s="7" r="H200">
-        <v>9529001</v>
+        <v>9529001.00</v>
       </c>
       <c s="7" r="I200">
         <v>20760.35</v>
@@ -9593,7 +9593,7 @@
         </is>
       </c>
       <c s="6" r="D201">
-        <v>425</v>
+        <v>425.00</v>
       </c>
       <c s="7" r="E201">
         <v>134956.12</v>
@@ -9614,7 +9614,7 @@
         <v>89.58</v>
       </c>
       <c s="7" r="K201">
-        <v>671992.8</v>
+        <v>671992.80</v>
       </c>
       <c s="7" r="L201">
         <v>1581.16</v>
@@ -9641,7 +9641,7 @@
         </is>
       </c>
       <c s="6" r="D202">
-        <v>499</v>
+        <v>499.00</v>
       </c>
       <c s="7" r="E202">
         <v>16639.67</v>
@@ -9689,7 +9689,7 @@
         </is>
       </c>
       <c s="6" r="D203">
-        <v>529</v>
+        <v>529.00</v>
       </c>
       <c s="7" r="E203">
         <v>113390.66</v>
@@ -9701,7 +9701,7 @@
         <v>1.35</v>
       </c>
       <c s="7" r="H203">
-        <v>8062421</v>
+        <v>8062421.00</v>
       </c>
       <c s="7" r="I203">
         <v>15240.87</v>
@@ -9719,7 +9719,7 @@
         <v>2.88</v>
       </c>
       <c s="7" r="N203">
-        <v>8418376.6</v>
+        <v>8418376.60</v>
       </c>
       <c s="7" r="O203">
         <v>15913.75</v>
@@ -9737,7 +9737,7 @@
         </is>
       </c>
       <c s="6" r="D204">
-        <v>430</v>
+        <v>430.00</v>
       </c>
       <c s="7" r="E204">
         <v>107166.89</v>
@@ -9746,10 +9746,10 @@
         <v>249.23</v>
       </c>
       <c s="7" r="G204">
-        <v>1.6</v>
+        <v>1.60</v>
       </c>
       <c s="7" r="H204">
-        <v>6388048</v>
+        <v>6388048.00</v>
       </c>
       <c s="7" r="I204">
         <v>14855.93</v>
@@ -9785,10 +9785,10 @@
         </is>
       </c>
       <c s="6" r="D205">
-        <v>311</v>
+        <v>311.00</v>
       </c>
       <c s="7" r="E205">
-        <v>460787</v>
+        <v>460787.00</v>
       </c>
       <c s="7" r="F205">
         <v>1481.63</v>
@@ -9797,7 +9797,7 @@
         <v>7.44</v>
       </c>
       <c s="7" r="H205">
-        <v>5403694</v>
+        <v>5403694.00</v>
       </c>
       <c s="7" r="I205">
         <v>17375.22</v>
@@ -9806,16 +9806,16 @@
         <v>87.26</v>
       </c>
       <c s="7" r="K205">
-        <v>328093</v>
+        <v>328093.00</v>
       </c>
       <c s="7" r="L205">
         <v>1054.96</v>
       </c>
       <c s="7" r="M205">
-        <v>5.3</v>
+        <v>5.30</v>
       </c>
       <c s="7" r="N205">
-        <v>6192574</v>
+        <v>6192574.00</v>
       </c>
       <c s="7" r="O205">
         <v>19911.81</v>
@@ -9833,10 +9833,10 @@
         </is>
       </c>
       <c s="6" r="D206">
-        <v>318</v>
+        <v>318.00</v>
       </c>
       <c s="7" r="E206">
-        <v>173550</v>
+        <v>173550.00</v>
       </c>
       <c s="7" r="F206">
         <v>545.75</v>
@@ -9845,7 +9845,7 @@
         <v>2.97</v>
       </c>
       <c s="7" r="H206">
-        <v>5377309</v>
+        <v>5377309.00</v>
       </c>
       <c s="7" r="I206">
         <v>16909.78</v>
@@ -9854,16 +9854,16 @@
         <v>92.03</v>
       </c>
       <c s="7" r="K206">
-        <v>292420</v>
+        <v>292420.00</v>
       </c>
       <c s="7" r="L206">
         <v>919.56</v>
       </c>
       <c s="7" r="M206">
-        <v>5</v>
+        <v>5.00</v>
       </c>
       <c s="7" r="N206">
-        <v>5843279</v>
+        <v>5843279.00</v>
       </c>
       <c s="7" r="O206">
         <v>18375.09</v>
@@ -9881,7 +9881,7 @@
         </is>
       </c>
       <c s="6" r="D207">
-        <v>400</v>
+        <v>400.00</v>
       </c>
       <c s="7" r="E207">
         <v>822762.12</v>
@@ -9899,7 +9899,7 @@
         <v>13891.96</v>
       </c>
       <c s="7" r="J207">
-        <v>83</v>
+        <v>83.00</v>
       </c>
       <c s="7" r="K207">
         <v>315467.22</v>
@@ -9929,7 +9929,7 @@
         </is>
       </c>
       <c s="6" r="D208">
-        <v>551</v>
+        <v>551.00</v>
       </c>
       <c s="7" r="E208">
         <v>191154.02</v>
@@ -9941,13 +9941,13 @@
         <v>2.45</v>
       </c>
       <c s="7" r="H208">
-        <v>7432082</v>
+        <v>7432082.00</v>
       </c>
       <c s="7" r="I208">
         <v>13488.35</v>
       </c>
       <c s="7" r="J208">
-        <v>95.2</v>
+        <v>95.20</v>
       </c>
       <c s="7" r="K208">
         <v>183521.92</v>
@@ -9977,19 +9977,19 @@
         </is>
       </c>
       <c s="6" r="D209">
-        <v>336</v>
+        <v>336.00</v>
       </c>
       <c s="7" r="E209">
         <v>144883.04</v>
       </c>
       <c s="7" r="F209">
-        <v>431.2</v>
+        <v>431.20</v>
       </c>
       <c s="7" r="G209">
         <v>2.41</v>
       </c>
       <c s="7" r="H209">
-        <v>5354591</v>
+        <v>5354591.00</v>
       </c>
       <c s="7" r="I209">
         <v>15936.28</v>
@@ -10025,7 +10025,7 @@
         </is>
       </c>
       <c s="6" r="D210">
-        <v>277</v>
+        <v>277.00</v>
       </c>
       <c s="7" r="E210">
         <v>531159.38</v>
@@ -10037,13 +10037,13 @@
         <v>11.65</v>
       </c>
       <c s="7" r="H210">
-        <v>3869082</v>
+        <v>3869082.00</v>
       </c>
       <c s="7" r="I210">
         <v>13967.81</v>
       </c>
       <c s="7" r="J210">
-        <v>84.9</v>
+        <v>84.90</v>
       </c>
       <c s="7" r="K210">
         <v>157199.18</v>
@@ -10073,10 +10073,10 @@
         </is>
       </c>
       <c s="6" r="D211">
-        <v>222</v>
+        <v>222.00</v>
       </c>
       <c s="7" r="E211">
-        <v>56360</v>
+        <v>56360.00</v>
       </c>
       <c s="7" r="F211">
         <v>253.87</v>
@@ -10085,7 +10085,7 @@
         <v>1.54</v>
       </c>
       <c s="7" r="H211">
-        <v>3216729</v>
+        <v>3216729.00</v>
       </c>
       <c s="7" r="I211">
         <v>14489.77</v>
@@ -10094,7 +10094,7 @@
         <v>87.67</v>
       </c>
       <c s="7" r="K211">
-        <v>395945</v>
+        <v>395945.00</v>
       </c>
       <c s="7" r="L211">
         <v>1783.54</v>
@@ -10103,7 +10103,7 @@
         <v>10.79</v>
       </c>
       <c s="7" r="N211">
-        <v>3669034</v>
+        <v>3669034.00</v>
       </c>
       <c s="7" r="O211">
         <v>16527.18</v>
@@ -10121,7 +10121,7 @@
         </is>
       </c>
       <c s="6" r="D212">
-        <v>1825</v>
+        <v>1825.00</v>
       </c>
       <c s="7" r="E212">
         <v>670076.37</v>
@@ -10142,7 +10142,7 @@
         <v>95.64</v>
       </c>
       <c s="7" r="K212">
-        <v>504561.8</v>
+        <v>504561.80</v>
       </c>
       <c s="7" r="L212">
         <v>276.47</v>
@@ -10169,7 +10169,7 @@
         </is>
       </c>
       <c s="6" r="D213">
-        <v>472</v>
+        <v>472.00</v>
       </c>
       <c s="7" r="E213">
         <v>18522.85</v>
@@ -10181,7 +10181,7 @@
         <v>0.24</v>
       </c>
       <c s="7" r="H213">
-        <v>7008220</v>
+        <v>7008220.00</v>
       </c>
       <c s="7" r="I213">
         <v>14847.92</v>
@@ -10196,7 +10196,7 @@
         <v>1295.22</v>
       </c>
       <c s="7" r="M213">
-        <v>8</v>
+        <v>8.00</v>
       </c>
       <c s="7" r="N213">
         <v>7638086.57</v>
@@ -10217,7 +10217,7 @@
         </is>
       </c>
       <c s="6" r="D214">
-        <v>468</v>
+        <v>468.00</v>
       </c>
       <c s="7" r="E214">
         <v>317551.48</v>
@@ -10229,7 +10229,7 @@
         <v>4.43</v>
       </c>
       <c s="7" r="H214">
-        <v>6661835</v>
+        <v>6661835.00</v>
       </c>
       <c s="7" r="I214">
         <v>14234.69</v>
@@ -10265,7 +10265,7 @@
         </is>
       </c>
       <c s="6" r="D215">
-        <v>589</v>
+        <v>589.00</v>
       </c>
       <c s="7" r="E215">
         <v>162119.49</v>
@@ -10277,16 +10277,16 @@
         <v>1.73</v>
       </c>
       <c s="7" r="H215">
-        <v>8302486</v>
+        <v>8302486.00</v>
       </c>
       <c s="7" r="I215">
-        <v>14095.9</v>
+        <v>14095.90</v>
       </c>
       <c s="7" r="J215">
         <v>88.48</v>
       </c>
       <c s="7" r="K215">
-        <v>918889.6</v>
+        <v>918889.60</v>
       </c>
       <c s="7" r="L215">
         <v>1560.08</v>
@@ -10313,19 +10313,19 @@
         </is>
       </c>
       <c s="6" r="D216">
-        <v>225</v>
+        <v>225.00</v>
       </c>
       <c s="7" r="E216">
-        <v>2385450.9</v>
+        <v>2385450.90</v>
       </c>
       <c s="7" r="F216">
-        <v>10602</v>
+        <v>10602.00</v>
       </c>
       <c s="7" r="G216">
         <v>57.68</v>
       </c>
       <c s="7" r="H216">
-        <v>1282970</v>
+        <v>1282970.00</v>
       </c>
       <c s="7" r="I216">
         <v>5702.09</v>
@@ -10361,7 +10361,7 @@
         </is>
       </c>
       <c s="6" r="D217">
-        <v>679</v>
+        <v>679.00</v>
       </c>
       <c s="7" r="E217">
         <v>1075628.65</v>
@@ -10373,13 +10373,13 @@
         <v>8.99</v>
       </c>
       <c s="7" r="H217">
-        <v>9638596</v>
+        <v>9638596.00</v>
       </c>
       <c s="7" r="I217">
         <v>14195.28</v>
       </c>
       <c s="7" r="J217">
-        <v>80.6</v>
+        <v>80.60</v>
       </c>
       <c s="7" r="K217">
         <v>1244898.98</v>
@@ -10409,10 +10409,10 @@
         </is>
       </c>
       <c s="6" r="D218">
-        <v>911</v>
+        <v>911.00</v>
       </c>
       <c s="7" r="E218">
-        <v>150292</v>
+        <v>150292.00</v>
       </c>
       <c s="7" r="F218">
         <v>164.97</v>
@@ -10421,16 +10421,16 @@
         <v>1.05</v>
       </c>
       <c s="7" r="H218">
-        <v>12765845</v>
+        <v>12765845.00</v>
       </c>
       <c s="7" r="I218">
-        <v>14013</v>
+        <v>14013.00</v>
       </c>
       <c s="7" r="J218">
         <v>88.88</v>
       </c>
       <c s="7" r="K218">
-        <v>1447630</v>
+        <v>1447630.00</v>
       </c>
       <c s="7" r="L218">
         <v>1589.06</v>
@@ -10439,7 +10439,7 @@
         <v>10.08</v>
       </c>
       <c s="7" r="N218">
-        <v>14363767</v>
+        <v>14363767.00</v>
       </c>
       <c s="7" r="O218">
         <v>15767.03</v>
@@ -10457,10 +10457,10 @@
         </is>
       </c>
       <c s="6" r="D219">
-        <v>187</v>
+        <v>187.00</v>
       </c>
       <c s="7" r="E219">
-        <v>21101.9</v>
+        <v>21101.90</v>
       </c>
       <c s="7" r="F219">
         <v>112.84</v>
@@ -10469,7 +10469,7 @@
         <v>0.61</v>
       </c>
       <c s="7" r="H219">
-        <v>3090335</v>
+        <v>3090335.00</v>
       </c>
       <c s="7" r="I219">
         <v>16525.86</v>
@@ -10478,7 +10478,7 @@
         <v>89.46</v>
       </c>
       <c s="7" r="K219">
-        <v>343041</v>
+        <v>343041.00</v>
       </c>
       <c s="7" r="L219">
         <v>1834.44</v>
@@ -10487,7 +10487,7 @@
         <v>9.93</v>
       </c>
       <c s="7" r="N219">
-        <v>3454477.9</v>
+        <v>3454477.90</v>
       </c>
       <c s="7" r="O219">
         <v>18473.14</v>
@@ -10505,7 +10505,7 @@
         </is>
       </c>
       <c s="6" r="D220">
-        <v>386</v>
+        <v>386.00</v>
       </c>
       <c s="7" r="E220">
         <v>222616.95</v>
@@ -10532,7 +10532,7 @@
         <v>658.68</v>
       </c>
       <c s="7" r="M220">
-        <v>4.7</v>
+        <v>4.70</v>
       </c>
       <c s="7" r="N220">
         <v>5415261.95</v>
@@ -10553,7 +10553,7 @@
         </is>
       </c>
       <c s="6" r="D221">
-        <v>236</v>
+        <v>236.00</v>
       </c>
       <c s="7" r="E221">
         <v>1984864.01</v>
@@ -10580,7 +10580,7 @@
         <v>1121.81</v>
       </c>
       <c s="7" r="M221">
-        <v>7.1</v>
+        <v>7.10</v>
       </c>
       <c s="7" r="N221">
         <v>3727019.43</v>
@@ -10601,7 +10601,7 @@
         </is>
       </c>
       <c s="6" r="D222">
-        <v>810</v>
+        <v>810.00</v>
       </c>
       <c s="7" r="E222">
         <v>7478691.06</v>
@@ -10613,7 +10613,7 @@
         <v>57.96</v>
       </c>
       <c s="7" r="H222">
-        <v>5066101</v>
+        <v>5066101.00</v>
       </c>
       <c s="7" r="I222">
         <v>6254.45</v>
@@ -10649,7 +10649,7 @@
         </is>
       </c>
       <c s="6" r="D223">
-        <v>351</v>
+        <v>351.00</v>
       </c>
       <c s="7" r="E223">
         <v>1029599.96</v>
@@ -10661,10 +10661,10 @@
         <v>15.16</v>
       </c>
       <c s="7" r="H223">
-        <v>5231022</v>
+        <v>5231022.00</v>
       </c>
       <c s="7" r="I223">
-        <v>14903.2</v>
+        <v>14903.20</v>
       </c>
       <c s="7" r="J223">
         <v>77.03</v>
@@ -10697,7 +10697,7 @@
         </is>
       </c>
       <c s="6" r="D224">
-        <v>232</v>
+        <v>232.00</v>
       </c>
       <c s="7" r="E224">
         <v>259552.97</v>
@@ -10709,7 +10709,7 @@
         <v>6.74</v>
       </c>
       <c s="7" r="H224">
-        <v>3345084</v>
+        <v>3345084.00</v>
       </c>
       <c s="7" r="I224">
         <v>14418.47</v>
@@ -10730,7 +10730,7 @@
         <v>3853542.35</v>
       </c>
       <c s="7" r="O224">
-        <v>16610.1</v>
+        <v>16610.10</v>
       </c>
     </row>
     <row r="225" ht="14.4" customHeight="0">
@@ -10745,7 +10745,7 @@
         </is>
       </c>
       <c s="6" r="D225">
-        <v>256</v>
+        <v>256.00</v>
       </c>
       <c s="7" r="E225">
         <v>833937.26</v>
@@ -10757,7 +10757,7 @@
         <v>18.21</v>
       </c>
       <c s="7" r="H225">
-        <v>3553958</v>
+        <v>3553958.00</v>
       </c>
       <c s="7" r="I225">
         <v>13882.65</v>
@@ -10793,7 +10793,7 @@
         </is>
       </c>
       <c s="6" r="D226">
-        <v>129</v>
+        <v>129.00</v>
       </c>
       <c s="7" r="E226">
         <v>413476.72</v>
@@ -10802,10 +10802,10 @@
         <v>3205.25</v>
       </c>
       <c s="7" r="G226">
-        <v>16.2</v>
+        <v>16.20</v>
       </c>
       <c s="7" r="H226">
-        <v>1991888</v>
+        <v>1991888.00</v>
       </c>
       <c s="7" r="I226">
         <v>15440.99</v>
@@ -10841,7 +10841,7 @@
         </is>
       </c>
       <c s="6" r="D227">
-        <v>209</v>
+        <v>209.00</v>
       </c>
       <c s="7" r="E227">
         <v>268682.59</v>
@@ -10853,7 +10853,7 @@
         <v>7.83</v>
       </c>
       <c s="7" r="H227">
-        <v>2998128</v>
+        <v>2998128.00</v>
       </c>
       <c s="7" r="I227">
         <v>14345.11</v>
@@ -10862,7 +10862,7 @@
         <v>87.39</v>
       </c>
       <c s="7" r="K227">
-        <v>163913</v>
+        <v>163913.00</v>
       </c>
       <c s="7" r="L227">
         <v>784.27</v>
@@ -10889,13 +10889,13 @@
         </is>
       </c>
       <c s="6" r="D228">
-        <v>599</v>
+        <v>599.00</v>
       </c>
       <c s="8" t="str" r="E228"/>
       <c s="8" t="str" r="F228"/>
       <c s="8" t="str" r="G228"/>
       <c s="7" r="H228">
-        <v>5254237</v>
+        <v>5254237.00</v>
       </c>
       <c s="7" r="I228">
         <v>8771.68</v>
@@ -10931,7 +10931,7 @@
         </is>
       </c>
       <c s="6" r="D229">
-        <v>216</v>
+        <v>216.00</v>
       </c>
       <c s="7" r="E229">
         <v>160579.45</v>
@@ -10979,22 +10979,22 @@
         </is>
       </c>
       <c s="6" r="D230">
-        <v>207</v>
+        <v>207.00</v>
       </c>
       <c s="7" r="E230">
         <v>415531.89</v>
       </c>
       <c s="7" r="F230">
-        <v>2007.4</v>
+        <v>2007.40</v>
       </c>
       <c s="7" r="G230">
         <v>10.49</v>
       </c>
       <c s="7" r="H230">
-        <v>2739997.1</v>
+        <v>2739997.10</v>
       </c>
       <c s="7" r="I230">
-        <v>13236.7</v>
+        <v>13236.70</v>
       </c>
       <c s="7" r="J230">
         <v>69.15</v>
@@ -11009,7 +11009,7 @@
         <v>20.36</v>
       </c>
       <c s="7" r="N230">
-        <v>3962346.9</v>
+        <v>3962346.90</v>
       </c>
       <c s="7" r="O230">
         <v>19141.77</v>
@@ -11027,13 +11027,13 @@
         </is>
       </c>
       <c s="6" r="D231">
-        <v>207</v>
+        <v>207.00</v>
       </c>
       <c s="7" r="E231">
         <v>3077510.94</v>
       </c>
       <c s="7" r="F231">
-        <v>14867.2</v>
+        <v>14867.20</v>
       </c>
       <c s="7" r="G231">
         <v>96.53</v>
@@ -11051,7 +11051,7 @@
         <v>182450.59</v>
       </c>
       <c s="7" r="L231">
-        <v>881.4</v>
+        <v>881.40</v>
       </c>
       <c s="7" r="M231">
         <v>5.72</v>
@@ -11075,7 +11075,7 @@
         </is>
       </c>
       <c s="6" r="D232">
-        <v>145</v>
+        <v>145.00</v>
       </c>
       <c s="7" r="E232">
         <v>414914.94</v>
@@ -11087,7 +11087,7 @@
         <v>14.34</v>
       </c>
       <c s="7" r="H232">
-        <v>2159921</v>
+        <v>2159921.00</v>
       </c>
       <c s="7" r="I232">
         <v>14896.01</v>
@@ -11108,7 +11108,7 @@
         <v>2894243.76</v>
       </c>
       <c s="7" r="O232">
-        <v>19960.3</v>
+        <v>19960.30</v>
       </c>
     </row>
     <row r="233" ht="14.4" customHeight="0">
@@ -11123,7 +11123,7 @@
         </is>
       </c>
       <c s="6" r="D233">
-        <v>319</v>
+        <v>319.00</v>
       </c>
       <c s="7" r="E233">
         <v>225831.27</v>
@@ -11141,7 +11141,7 @@
         <v>22588.58</v>
       </c>
       <c s="7" r="J233">
-        <v>95.1</v>
+        <v>95.10</v>
       </c>
       <c s="7" r="K233">
         <v>145723.46</v>
@@ -11171,7 +11171,7 @@
         </is>
       </c>
       <c s="6" r="D234">
-        <v>88</v>
+        <v>88.00</v>
       </c>
       <c s="7" r="E234">
         <v>457427.47</v>
@@ -11183,7 +11183,7 @@
         <v>18.43</v>
       </c>
       <c s="7" r="H234">
-        <v>1150733</v>
+        <v>1150733.00</v>
       </c>
       <c s="7" r="I234">
         <v>13076.51</v>
@@ -11219,19 +11219,19 @@
         </is>
       </c>
       <c s="6" r="D235">
-        <v>47</v>
+        <v>47.00</v>
       </c>
       <c s="7" r="E235">
         <v>104297.55</v>
       </c>
       <c s="7" r="F235">
-        <v>2219.1</v>
+        <v>2219.10</v>
       </c>
       <c s="7" r="G235">
         <v>10.99</v>
       </c>
       <c s="7" r="H235">
-        <v>734067</v>
+        <v>734067.00</v>
       </c>
       <c s="7" r="I235">
         <v>15618.45</v>
@@ -11249,7 +11249,7 @@
         <v>11.69</v>
       </c>
       <c s="7" r="N235">
-        <v>949327.3</v>
+        <v>949327.30</v>
       </c>
       <c s="7" r="O235">
         <v>20198.46</v>
@@ -11267,7 +11267,7 @@
         </is>
       </c>
       <c s="6" r="D236">
-        <v>1211</v>
+        <v>1211.00</v>
       </c>
       <c s="7" r="E236">
         <v>1385947.12</v>
@@ -11282,13 +11282,13 @@
         <v>15585931.44</v>
       </c>
       <c s="7" r="I236">
-        <v>12870.3</v>
+        <v>12870.30</v>
       </c>
       <c s="7" r="J236">
         <v>82.94</v>
       </c>
       <c s="7" r="K236">
-        <v>1820703.9</v>
+        <v>1820703.90</v>
       </c>
       <c s="7" r="L236">
         <v>1503.47</v>
@@ -11315,13 +11315,13 @@
         </is>
       </c>
       <c s="6" r="D237">
-        <v>6446</v>
+        <v>6446.00</v>
       </c>
       <c s="7" r="E237">
         <v>33767352.38</v>
       </c>
       <c s="7" r="F237">
-        <v>5238.5</v>
+        <v>5238.50</v>
       </c>
       <c s="7" r="G237">
         <v>33.98</v>
@@ -11330,7 +11330,7 @@
         <v>56026700.83</v>
       </c>
       <c s="7" r="I237">
-        <v>8691.7</v>
+        <v>8691.70</v>
       </c>
       <c s="7" r="J237">
         <v>56.38</v>
@@ -11363,7 +11363,7 @@
         </is>
       </c>
       <c s="6" r="D238">
-        <v>1952</v>
+        <v>1952.00</v>
       </c>
       <c s="7" r="E238">
         <v>8808929.64</v>
@@ -11411,7 +11411,7 @@
         </is>
       </c>
       <c s="6" r="D239">
-        <v>2490</v>
+        <v>2490.00</v>
       </c>
       <c s="7" r="E239">
         <v>16538344.28</v>
@@ -11426,7 +11426,7 @@
         <v>18884652.82</v>
       </c>
       <c s="7" r="I239">
-        <v>7584.2</v>
+        <v>7584.20</v>
       </c>
       <c s="7" r="J239">
         <v>47.99</v>
@@ -11459,13 +11459,13 @@
         </is>
       </c>
       <c s="6" r="D240">
-        <v>1198</v>
+        <v>1198.00</v>
       </c>
       <c s="7" r="E240">
         <v>2211870.38</v>
       </c>
       <c s="7" r="F240">
-        <v>1846.3</v>
+        <v>1846.30</v>
       </c>
       <c s="7" r="G240">
         <v>11.66</v>
@@ -11489,7 +11489,7 @@
         <v>3.86</v>
       </c>
       <c s="7" r="N240">
-        <v>18968011.3</v>
+        <v>18968011.30</v>
       </c>
       <c s="7" r="O240">
         <v>15833.06</v>
@@ -11507,7 +11507,7 @@
         </is>
       </c>
       <c s="6" r="D241">
-        <v>8107</v>
+        <v>8107.00</v>
       </c>
       <c s="7" r="E241">
         <v>38972870.41</v>
@@ -11555,7 +11555,7 @@
         </is>
       </c>
       <c s="6" r="D242">
-        <v>2165</v>
+        <v>2165.00</v>
       </c>
       <c s="7" r="E242">
         <v>8282115.78</v>
@@ -11573,7 +11573,7 @@
         <v>8687.63</v>
       </c>
       <c s="7" r="J242">
-        <v>62.5</v>
+        <v>62.50</v>
       </c>
       <c s="7" r="K242">
         <v>3004195.31</v>
@@ -11610,16 +11610,16 @@
         <v>6975.96243358363</v>
       </c>
       <c s="7" r="G243">
-        <v>44.2411485323007</v>
+        <v>43.5262681844772</v>
       </c>
       <c s="7" r="H243">
         <v>13545123078.79</v>
       </c>
       <c s="7" r="I243">
-        <v>7764.02790255072</v>
+        <v>7764.02790255073</v>
       </c>
       <c s="7" r="J243">
-        <v>49.2390139591419</v>
+        <v>49.911162709837</v>
       </c>
       <c s="7" r="K243">
         <v>1793537165.07</v>
@@ -11631,10 +11631,10 @@
         <v>6.5198375085574</v>
       </c>
       <c s="7" r="N243">
-        <v>27508924305.49</v>
+        <v>27514534758.12</v>
       </c>
       <c s="7" r="O243">
-        <v>15768.0409867534</v>
+        <v>15771.256883021896136650235011</v>
       </c>
     </row>
     <row r="244" ht="3.05" customHeight="1"/>

</xml_diff>